<commit_message>
Test 42 - group rejoin after zoning, aggro wipe on death, personal heal messages, window positions, pet titles
 - Threat stickiness (10% to switch, taunt overrides), Auto-Loot on Kill option
  - Kenji tail tip, troll run shoulders (tools/relax_shoulders.gd)
  - Lightmender Spiritual Weapon level 1 starting spell at 40% health, holds no gear; 14 characters per account
  - Player-lit campfires from Firewood Bundles (campfire_relay.gd), tiered regen and XP bonus
  - Respawn timers start at death, 6x longer common timers, no spawns within 12 m of a player; Halvek in the mausoleum
  - EQ-style fear on players: save roll decides Shaken (stat loss) or Terrified (run blindly); Lizardkin fear save live
  - Fix freed-target errors in pet assist and macros
  - test_test42, docs, manual
</commit_message>
<xml_diff>
--- a/Data/player_spells.xlsx
+++ b/Data/player_spells.xlsx
@@ -13037,11 +13037,11 @@
       </c>
       <c r="C134" s="12" t="inlineStr">
         <is>
-          <t>Summons weapon (30% caster's damage) for 15 seconds (D&amp;D-inspired).</t>
+          <t>Summons a spiritual weapon with 40% of your health that fights at your side until destroyed.</t>
         </is>
       </c>
       <c r="D134" s="11" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E134" s="12" t="inlineStr">
         <is>
@@ -13113,7 +13113,7 @@
       </c>
       <c r="Y134" s="12" t="inlineStr">
         <is>
-          <t>Lightmender:7</t>
+          <t>Lightmender:1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
crime system, fixed art issues with jumping and large races, began work on lumora
  - Crime and the courthouse: PvP in town is a crime, guards demand the fine (pay or resist), Magistrate
  - Lumora stand-ins: district buildings, 14 trainers with class scrolls, inn, temple healer, crier, notice board, Ralph's Last Round
  - Shadowblade: stealth hides from monsters and shows (faint + [stealth]), stealth icon, physical skills instant/no mana, Blindside stun; stuns hold monsters still
  - Cross-zone group health bars, /ban by name across zones, follow says who left
  - Summoned animal pets move like critters; troll/ogre female running hump
  - cast_message field on every spell; starting spells granted to older characters
</commit_message>
<xml_diff>
--- a/Data/player_spells.xlsx
+++ b/Data/player_spells.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Y561"/>
+  <dimension ref="A1:Z562"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="15.3" customWidth="1" style="8" min="1" max="1"/>
@@ -593,6 +593,11 @@
           <t>class_level_requirements</t>
         </is>
       </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>cast_message</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="23.85" customHeight="1" s="9">
       <c r="A2" s="11" t="n">
@@ -688,6 +693,7 @@
           <t>Voidknight:1</t>
         </is>
       </c>
+      <c r="Z2" t="inlineStr"/>
     </row>
     <row r="3" ht="23.85" customHeight="1" s="9">
       <c r="A3" s="13" t="n">
@@ -783,6 +789,7 @@
           <t>Voidknight:1</t>
         </is>
       </c>
+      <c r="Z3" t="inlineStr"/>
     </row>
     <row r="4" ht="15" customHeight="1" s="9">
       <c r="A4" s="11" t="n">
@@ -878,6 +885,7 @@
           <t>Voidknight:2</t>
         </is>
       </c>
+      <c r="Z4" t="inlineStr"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="9">
       <c r="A5" s="13" t="n">
@@ -973,6 +981,7 @@
           <t>Voidknight:2</t>
         </is>
       </c>
+      <c r="Z5" t="inlineStr"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="9">
       <c r="A6" s="11" t="n">
@@ -1064,6 +1073,7 @@
           <t>Blademaster:7, Voidknight:3</t>
         </is>
       </c>
+      <c r="Z6" t="inlineStr"/>
     </row>
     <row r="7" ht="15" customHeight="1" s="9">
       <c r="A7" s="13" t="n">
@@ -1161,6 +1171,7 @@
           <t>Voidknight:3</t>
         </is>
       </c>
+      <c r="Z7" t="inlineStr"/>
     </row>
     <row r="8" ht="23.85" customHeight="1" s="9">
       <c r="A8" s="11" t="n">
@@ -1256,6 +1267,7 @@
           <t>Voidknight:4</t>
         </is>
       </c>
+      <c r="Z8" t="inlineStr"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="9">
       <c r="A9" s="13" t="n">
@@ -1351,6 +1363,7 @@
           <t>Voidknight:4</t>
         </is>
       </c>
+      <c r="Z9" t="inlineStr"/>
     </row>
     <row r="10" ht="23.85" customHeight="1" s="9">
       <c r="A10" s="11" t="n">
@@ -1442,6 +1455,7 @@
           <t>Voidknight:5</t>
         </is>
       </c>
+      <c r="Z10" t="inlineStr"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="9">
       <c r="A11" s="13" t="n">
@@ -1630,6 +1644,7 @@
           <t>Voidknight:6</t>
         </is>
       </c>
+      <c r="Z12" t="inlineStr"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="13" t="n">
@@ -1725,6 +1740,7 @@
           <t>Voidknight:6</t>
         </is>
       </c>
+      <c r="Z13" t="inlineStr"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="9">
       <c r="A14" s="11" t="n">
@@ -1816,6 +1832,7 @@
           <t>Blademaster:3, Voidknight:7</t>
         </is>
       </c>
+      <c r="Z14" t="inlineStr"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="9">
       <c r="A15" s="13" t="n">
@@ -2006,6 +2023,7 @@
           <t>Voidknight:8</t>
         </is>
       </c>
+      <c r="Z16" t="inlineStr"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="9">
       <c r="A17" s="13" t="n">
@@ -2101,6 +2119,7 @@
           <t>Voidknight:8</t>
         </is>
       </c>
+      <c r="Z17" t="inlineStr"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="9">
       <c r="A18" s="11" t="n">
@@ -2196,6 +2215,7 @@
           <t>Voidknight:9</t>
         </is>
       </c>
+      <c r="Z18" t="inlineStr"/>
     </row>
     <row r="19" ht="15" customHeight="1" s="9">
       <c r="A19" s="13" t="n">
@@ -2291,6 +2311,7 @@
           <t>Voidknight:9</t>
         </is>
       </c>
+      <c r="Z19" t="inlineStr"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="9">
       <c r="A20" s="11" t="n">
@@ -2384,6 +2405,7 @@
           <t>Blademaster:10, Voidknight:10</t>
         </is>
       </c>
+      <c r="Z20" t="inlineStr"/>
     </row>
     <row r="21" ht="23.85" customHeight="1" s="9">
       <c r="A21" s="13" t="n">
@@ -2481,6 +2503,7 @@
           <t>Voidknight:10</t>
         </is>
       </c>
+      <c r="Z21" t="inlineStr"/>
     </row>
     <row r="22" ht="23.85" customHeight="1" s="9">
       <c r="A22" s="11" t="n">
@@ -2578,6 +2601,7 @@
           <t>Voidknight:11</t>
         </is>
       </c>
+      <c r="Z22" t="inlineStr"/>
     </row>
     <row r="23" ht="23.85" customHeight="1" s="9">
       <c r="A23" s="13" t="n">
@@ -2673,6 +2697,7 @@
           <t>Voidknight:11</t>
         </is>
       </c>
+      <c r="Z23" t="inlineStr"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="9">
       <c r="A24" s="11" t="n">
@@ -2768,6 +2793,7 @@
           <t>Voidknight:12</t>
         </is>
       </c>
+      <c r="Z24" t="inlineStr"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="9">
       <c r="A25" s="13" t="n">
@@ -2863,6 +2889,7 @@
           <t>Voidknight:12</t>
         </is>
       </c>
+      <c r="Z25" t="inlineStr"/>
     </row>
     <row r="26" ht="23.85" customHeight="1" s="9">
       <c r="A26" s="11" t="n">
@@ -2960,6 +2987,7 @@
           <t>Voidknight:13</t>
         </is>
       </c>
+      <c r="Z26" t="inlineStr"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="9">
       <c r="A27" s="13" t="n">
@@ -3051,6 +3079,7 @@
           <t>Voidknight:13</t>
         </is>
       </c>
+      <c r="Z27" t="inlineStr"/>
     </row>
     <row r="28" ht="23.85" customHeight="1" s="9">
       <c r="A28" s="11" t="n">
@@ -3146,6 +3175,7 @@
           <t>Lightsworn:10, Voidknight:14</t>
         </is>
       </c>
+      <c r="Z28" t="inlineStr"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="9">
       <c r="A29" s="13" t="n">
@@ -3338,6 +3368,7 @@
           <t>Voidknight:15</t>
         </is>
       </c>
+      <c r="Z30" t="inlineStr"/>
     </row>
     <row r="31" ht="15" customHeight="1" s="9">
       <c r="A31" s="13" t="n">
@@ -3435,6 +3466,7 @@
           <t>Voidknight:15</t>
         </is>
       </c>
+      <c r="Z31" t="inlineStr"/>
     </row>
     <row r="32" ht="15" customHeight="1" s="9">
       <c r="A32" s="11" t="n">
@@ -3530,6 +3562,7 @@
           <t>Voidknight:16</t>
         </is>
       </c>
+      <c r="Z32" t="inlineStr"/>
     </row>
     <row r="33" ht="15" customHeight="1" s="9">
       <c r="A33" s="13" t="n">
@@ -3629,6 +3662,7 @@
           <t>Voidknight:16</t>
         </is>
       </c>
+      <c r="Z33" t="inlineStr"/>
     </row>
     <row r="34" ht="23.85" customHeight="1" s="9">
       <c r="A34" s="11" t="n">
@@ -3720,6 +3754,7 @@
           <t>Voidknight:17</t>
         </is>
       </c>
+      <c r="Z34" t="inlineStr"/>
     </row>
     <row r="35" ht="15" customHeight="1" s="9">
       <c r="A35" s="13" t="n">
@@ -3815,6 +3850,7 @@
           <t>Voidknight:17</t>
         </is>
       </c>
+      <c r="Z35" t="inlineStr"/>
     </row>
     <row r="36" ht="15" customHeight="1" s="9">
       <c r="A36" s="11" t="n">
@@ -3910,6 +3946,7 @@
           <t>Voidknight:18</t>
         </is>
       </c>
+      <c r="Z36" t="inlineStr"/>
     </row>
     <row r="37" ht="23.85" customHeight="1" s="9">
       <c r="A37" s="13" t="n">
@@ -4007,6 +4044,7 @@
           <t>Voidknight:18</t>
         </is>
       </c>
+      <c r="Z37" t="inlineStr"/>
     </row>
     <row r="38" ht="15" customHeight="1" s="9">
       <c r="A38" s="11" t="n">
@@ -4102,6 +4140,7 @@
           <t>Voidknight:19</t>
         </is>
       </c>
+      <c r="Z38" t="inlineStr"/>
     </row>
     <row r="39" ht="15" customHeight="1" s="9">
       <c r="A39" s="13" t="n">
@@ -4197,6 +4236,7 @@
           <t>Voidknight:19</t>
         </is>
       </c>
+      <c r="Z39" t="inlineStr"/>
     </row>
     <row r="40" ht="23.85" customHeight="1" s="9">
       <c r="A40" s="11" t="n">
@@ -4292,6 +4332,7 @@
           <t>Voidknight:20</t>
         </is>
       </c>
+      <c r="Z40" t="inlineStr"/>
     </row>
     <row r="41" ht="23.85" customHeight="1" s="9">
       <c r="A41" s="13" t="n">
@@ -4387,6 +4428,7 @@
           <t>Voidknight:20</t>
         </is>
       </c>
+      <c r="Z41" t="inlineStr"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="9">
       <c r="A42" s="11" t="n">
@@ -4482,6 +4524,7 @@
           <t>Voidknight:20</t>
         </is>
       </c>
+      <c r="Z42" t="inlineStr"/>
     </row>
     <row r="43" ht="15" customHeight="1" s="9">
       <c r="A43" s="13" t="n">
@@ -4573,6 +4616,7 @@
           <t>Lightsworn:1</t>
         </is>
       </c>
+      <c r="Z43" t="inlineStr"/>
     </row>
     <row r="44" ht="15" customHeight="1" s="9">
       <c r="A44" s="11" t="n">
@@ -4670,6 +4714,7 @@
           <t>Lightsworn:1</t>
         </is>
       </c>
+      <c r="Z44" t="inlineStr"/>
     </row>
     <row r="45" ht="15" customHeight="1" s="9">
       <c r="A45" s="13" t="n">
@@ -4765,6 +4810,7 @@
           <t>Lightsworn:2</t>
         </is>
       </c>
+      <c r="Z45" t="inlineStr"/>
     </row>
     <row r="46" ht="15" customHeight="1" s="9">
       <c r="A46" s="11" t="n">
@@ -4856,6 +4902,7 @@
           <t>Lightsworn:2</t>
         </is>
       </c>
+      <c r="Z46" t="inlineStr"/>
     </row>
     <row r="47" ht="15" customHeight="1" s="9">
       <c r="A47" s="13" t="n">
@@ -4947,6 +4994,7 @@
           <t>Lightsworn:3, Zenblade:7</t>
         </is>
       </c>
+      <c r="Z47" t="inlineStr"/>
     </row>
     <row r="48" ht="15" customHeight="1" s="9">
       <c r="A48" s="11" t="n">
@@ -5038,6 +5086,7 @@
           <t>Lightsworn:3</t>
         </is>
       </c>
+      <c r="Z48" t="inlineStr"/>
     </row>
     <row r="49" ht="15" customHeight="1" s="9">
       <c r="A49" s="13" t="n">
@@ -5133,6 +5182,7 @@
           <t>Lightsworn:4</t>
         </is>
       </c>
+      <c r="Z49" t="inlineStr"/>
     </row>
     <row r="50" ht="15" customHeight="1" s="9">
       <c r="A50" s="11" t="n">
@@ -5224,6 +5274,7 @@
           <t>Lightsworn:4</t>
         </is>
       </c>
+      <c r="Z50" t="inlineStr"/>
     </row>
     <row r="51" ht="15" customHeight="1" s="9">
       <c r="A51" s="13" t="n">
@@ -5319,6 +5370,7 @@
           <t>Lightsworn:5</t>
         </is>
       </c>
+      <c r="Z51" t="inlineStr"/>
     </row>
     <row r="52" ht="15" customHeight="1" s="9">
       <c r="A52" s="11" t="n">
@@ -5414,6 +5466,7 @@
           <t>Lightsworn:5</t>
         </is>
       </c>
+      <c r="Z52" t="inlineStr"/>
     </row>
     <row r="53" ht="15" customHeight="1" s="9">
       <c r="A53" s="13" t="n">
@@ -5505,6 +5558,7 @@
           <t>Lightsworn:6</t>
         </is>
       </c>
+      <c r="Z53" t="inlineStr"/>
     </row>
     <row r="54" ht="15" customHeight="1" s="9">
       <c r="A54" s="11" t="n">
@@ -5602,6 +5656,7 @@
           <t>Lightsworn:6</t>
         </is>
       </c>
+      <c r="Z54" t="inlineStr"/>
     </row>
     <row r="55" ht="15" customHeight="1" s="9">
       <c r="A55" s="13" t="n">
@@ -5697,6 +5752,7 @@
           <t>Lightsworn:7</t>
         </is>
       </c>
+      <c r="Z55" t="inlineStr"/>
     </row>
     <row r="56" ht="15" customHeight="1" s="9">
       <c r="A56" s="11" t="n">
@@ -5792,6 +5848,7 @@
           <t>Lightsworn:7</t>
         </is>
       </c>
+      <c r="Z56" t="inlineStr"/>
     </row>
     <row r="57" ht="15" customHeight="1" s="9">
       <c r="A57" s="13" t="n">
@@ -5883,6 +5940,7 @@
           <t>Lightsworn:8</t>
         </is>
       </c>
+      <c r="Z57" t="inlineStr"/>
     </row>
     <row r="58" ht="15" customHeight="1" s="9">
       <c r="A58" s="11" t="n">
@@ -5978,6 +6036,7 @@
           <t>Lightsworn:8</t>
         </is>
       </c>
+      <c r="Z58" t="inlineStr"/>
     </row>
     <row r="59" ht="15" customHeight="1" s="9">
       <c r="A59" s="13" t="n">
@@ -6069,6 +6128,7 @@
           <t>Lightsworn:9</t>
         </is>
       </c>
+      <c r="Z59" t="inlineStr"/>
     </row>
     <row r="60" ht="15" customHeight="1" s="9">
       <c r="A60" s="11" t="n">
@@ -6160,6 +6220,7 @@
           <t>Lightsworn:9</t>
         </is>
       </c>
+      <c r="Z60" t="inlineStr"/>
     </row>
     <row r="61" ht="15" customHeight="1" s="9">
       <c r="A61" s="13" t="n">
@@ -6255,6 +6316,7 @@
           <t>Lightsworn:10</t>
         </is>
       </c>
+      <c r="Z61" t="inlineStr"/>
     </row>
     <row r="62" ht="15" customHeight="1" s="9">
       <c r="A62" s="11" t="n">
@@ -6346,6 +6408,7 @@
           <t>Lightsworn:11</t>
         </is>
       </c>
+      <c r="Z62" t="inlineStr"/>
     </row>
     <row r="63" ht="15" customHeight="1" s="9">
       <c r="A63" s="13" t="n">
@@ -6441,6 +6504,7 @@
           <t>Lightsworn:11</t>
         </is>
       </c>
+      <c r="Z63" t="inlineStr"/>
     </row>
     <row r="64" ht="15" customHeight="1" s="9">
       <c r="A64" s="11" t="n">
@@ -6536,6 +6600,7 @@
           <t>Lightsworn:12</t>
         </is>
       </c>
+      <c r="Z64" t="inlineStr"/>
     </row>
     <row r="65" ht="15" customHeight="1" s="9">
       <c r="A65" s="13" t="n">
@@ -6627,6 +6692,7 @@
           <t>Lightsworn:12</t>
         </is>
       </c>
+      <c r="Z65" t="inlineStr"/>
     </row>
     <row r="66" ht="23.85" customHeight="1" s="9">
       <c r="A66" s="11" t="n">
@@ -6722,6 +6788,7 @@
           <t>Lightsworn:13</t>
         </is>
       </c>
+      <c r="Z66" t="inlineStr"/>
     </row>
     <row r="67" ht="15" customHeight="1" s="9">
       <c r="A67" s="13" t="n">
@@ -6817,6 +6884,7 @@
           <t>Lightsworn:13</t>
         </is>
       </c>
+      <c r="Z67" t="inlineStr"/>
     </row>
     <row r="68" ht="15" customHeight="1" s="9">
       <c r="A68" s="11" t="n">
@@ -6908,6 +6976,7 @@
           <t>Lightsworn:14</t>
         </is>
       </c>
+      <c r="Z68" t="inlineStr"/>
     </row>
     <row r="69" ht="15" customHeight="1" s="9">
       <c r="A69" s="13" t="n">
@@ -6999,6 +7068,7 @@
           <t>Lightsworn:14</t>
         </is>
       </c>
+      <c r="Z69" t="inlineStr"/>
     </row>
     <row r="70" ht="15" customHeight="1" s="9">
       <c r="A70" s="11" t="n">
@@ -7094,6 +7164,7 @@
           <t>Lightsworn:15</t>
         </is>
       </c>
+      <c r="Z70" t="inlineStr"/>
     </row>
     <row r="71" ht="15" customHeight="1" s="9">
       <c r="A71" s="13" t="n">
@@ -7189,6 +7260,7 @@
           <t>Lightsworn:15</t>
         </is>
       </c>
+      <c r="Z71" t="inlineStr"/>
     </row>
     <row r="72" ht="15" customHeight="1" s="9">
       <c r="A72" s="11" t="n">
@@ -7284,6 +7356,7 @@
           <t>Lightsworn:16</t>
         </is>
       </c>
+      <c r="Z72" t="inlineStr"/>
     </row>
     <row r="73" ht="15" customHeight="1" s="9">
       <c r="A73" s="13" t="n">
@@ -7381,6 +7454,7 @@
           <t>Lightsworn:16</t>
         </is>
       </c>
+      <c r="Z73" t="inlineStr"/>
     </row>
     <row r="74" ht="15" customHeight="1" s="9">
       <c r="A74" s="11" t="n">
@@ -7476,6 +7550,7 @@
           <t>Lightsworn:17</t>
         </is>
       </c>
+      <c r="Z74" t="inlineStr"/>
     </row>
     <row r="75" ht="15" customHeight="1" s="9">
       <c r="A75" s="13" t="n">
@@ -7571,6 +7646,7 @@
           <t>Lightsworn:17</t>
         </is>
       </c>
+      <c r="Z75" t="inlineStr"/>
     </row>
     <row r="76" ht="15" customHeight="1" s="9">
       <c r="A76" s="11" t="n">
@@ -7761,6 +7837,7 @@
           <t>Lightsworn:18</t>
         </is>
       </c>
+      <c r="Z77" t="inlineStr"/>
     </row>
     <row r="78" ht="15" customHeight="1" s="9">
       <c r="A78" s="11" t="n">
@@ -7856,6 +7933,7 @@
           <t>Lightsworn:19</t>
         </is>
       </c>
+      <c r="Z78" t="inlineStr"/>
     </row>
     <row r="79" ht="15" customHeight="1" s="9">
       <c r="A79" s="13" t="n">
@@ -7947,6 +8025,7 @@
           <t>Lightsworn:19</t>
         </is>
       </c>
+      <c r="Z79" t="inlineStr"/>
     </row>
     <row r="80" ht="15" customHeight="1" s="9">
       <c r="A80" s="11" t="n">
@@ -8042,6 +8121,7 @@
           <t>Lightsworn:20</t>
         </is>
       </c>
+      <c r="Z80" t="inlineStr"/>
     </row>
     <row r="81" ht="15" customHeight="1" s="9">
       <c r="A81" s="13" t="n">
@@ -8137,6 +8217,7 @@
           <t>Lightsworn:20</t>
         </is>
       </c>
+      <c r="Z81" t="inlineStr"/>
     </row>
     <row r="82" ht="15" customHeight="1" s="9">
       <c r="A82" s="11" t="n">
@@ -8232,6 +8313,7 @@
           <t>Lightsworn:20</t>
         </is>
       </c>
+      <c r="Z82" t="inlineStr"/>
     </row>
     <row r="83" ht="15" customHeight="1" s="9">
       <c r="A83" s="13" t="n">
@@ -8323,6 +8405,7 @@
           <t>Blademaster:1</t>
         </is>
       </c>
+      <c r="Z83" t="inlineStr"/>
     </row>
     <row r="84" ht="15" customHeight="1" s="9">
       <c r="A84" s="11" t="n">
@@ -8414,6 +8497,7 @@
           <t>Blademaster:1</t>
         </is>
       </c>
+      <c r="Z84" t="inlineStr"/>
     </row>
     <row r="85" ht="15" customHeight="1" s="9">
       <c r="A85" s="13" t="n">
@@ -8509,6 +8593,7 @@
           <t>Blademaster:2</t>
         </is>
       </c>
+      <c r="Z85" t="inlineStr"/>
     </row>
     <row r="86" ht="15" customHeight="1" s="9">
       <c r="A86" s="11" t="n">
@@ -8600,6 +8685,7 @@
           <t>Blademaster:2</t>
         </is>
       </c>
+      <c r="Z86" t="inlineStr"/>
     </row>
     <row r="87" ht="15" customHeight="1" s="9">
       <c r="A87" s="13" t="n">
@@ -8695,6 +8781,7 @@
           <t>Blademaster:3</t>
         </is>
       </c>
+      <c r="Z87" t="inlineStr"/>
     </row>
     <row r="88" ht="15" customHeight="1" s="9">
       <c r="A88" s="11" t="n">
@@ -8790,6 +8877,7 @@
           <t>Blademaster:4</t>
         </is>
       </c>
+      <c r="Z88" t="inlineStr"/>
     </row>
     <row r="89" ht="15" customHeight="1" s="9">
       <c r="A89" s="13" t="n">
@@ -8881,6 +8969,7 @@
           <t>Blademaster:4</t>
         </is>
       </c>
+      <c r="Z89" t="inlineStr"/>
     </row>
     <row r="90" ht="15" customHeight="1" s="9">
       <c r="A90" s="11" t="n">
@@ -8976,6 +9065,7 @@
           <t>Blademaster:5</t>
         </is>
       </c>
+      <c r="Z90" t="inlineStr"/>
     </row>
     <row r="91" ht="15" customHeight="1" s="9">
       <c r="A91" s="13" t="n">
@@ -9071,6 +9161,7 @@
           <t>Blademaster:5</t>
         </is>
       </c>
+      <c r="Z91" t="inlineStr"/>
     </row>
     <row r="92" ht="15" customHeight="1" s="9">
       <c r="A92" s="11" t="n">
@@ -9166,6 +9257,7 @@
           <t>Blademaster:6</t>
         </is>
       </c>
+      <c r="Z92" t="inlineStr"/>
     </row>
     <row r="93" ht="15" customHeight="1" s="9">
       <c r="A93" s="13" t="n">
@@ -9261,6 +9353,7 @@
           <t>Blademaster:6</t>
         </is>
       </c>
+      <c r="Z93" t="inlineStr"/>
     </row>
     <row r="94" ht="15" customHeight="1" s="9">
       <c r="A94" s="11" t="n">
@@ -9356,6 +9449,7 @@
           <t>Blademaster:7</t>
         </is>
       </c>
+      <c r="Z94" t="inlineStr"/>
     </row>
     <row r="95" ht="15" customHeight="1" s="9">
       <c r="A95" s="13" t="n">
@@ -9447,6 +9541,7 @@
           <t>Blademaster:8</t>
         </is>
       </c>
+      <c r="Z95" t="inlineStr"/>
     </row>
     <row r="96" ht="15" customHeight="1" s="9">
       <c r="A96" s="11" t="n">
@@ -9542,6 +9637,7 @@
           <t>Blademaster:8</t>
         </is>
       </c>
+      <c r="Z96" t="inlineStr"/>
     </row>
     <row r="97" ht="15" customHeight="1" s="9">
       <c r="A97" s="13" t="n">
@@ -9637,6 +9733,7 @@
           <t>Blademaster:9</t>
         </is>
       </c>
+      <c r="Z97" t="inlineStr"/>
     </row>
     <row r="98" ht="15" customHeight="1" s="9">
       <c r="A98" s="11" t="n">
@@ -9728,6 +9825,7 @@
           <t>Blademaster:9</t>
         </is>
       </c>
+      <c r="Z98" t="inlineStr"/>
     </row>
     <row r="99" ht="15" customHeight="1" s="9">
       <c r="A99" s="13" t="n">
@@ -9823,6 +9921,7 @@
           <t>Blademaster:10</t>
         </is>
       </c>
+      <c r="Z99" t="inlineStr"/>
     </row>
     <row r="100" ht="15" customHeight="1" s="9">
       <c r="A100" s="11" t="n">
@@ -9920,6 +10019,7 @@
           <t>Blademaster:11</t>
         </is>
       </c>
+      <c r="Z100" t="inlineStr"/>
     </row>
     <row r="101" ht="15" customHeight="1" s="9">
       <c r="A101" s="13" t="n">
@@ -10017,6 +10117,7 @@
           <t>Blademaster:11</t>
         </is>
       </c>
+      <c r="Z101" t="inlineStr"/>
     </row>
     <row r="102" ht="15" customHeight="1" s="9">
       <c r="A102" s="11" t="n">
@@ -10108,6 +10209,7 @@
           <t>Blademaster:12</t>
         </is>
       </c>
+      <c r="Z102" t="inlineStr"/>
     </row>
     <row r="103" ht="15" customHeight="1" s="9">
       <c r="A103" s="13" t="n">
@@ -10199,6 +10301,7 @@
           <t>Blademaster:12</t>
         </is>
       </c>
+      <c r="Z103" t="inlineStr"/>
     </row>
     <row r="104" ht="15" customHeight="1" s="9">
       <c r="A104" s="11" t="n">
@@ -10290,6 +10393,7 @@
           <t>Blademaster:13</t>
         </is>
       </c>
+      <c r="Z104" t="inlineStr"/>
     </row>
     <row r="105" ht="15" customHeight="1" s="9">
       <c r="A105" s="13" t="n">
@@ -10381,6 +10485,7 @@
           <t>Blademaster:13</t>
         </is>
       </c>
+      <c r="Z105" t="inlineStr"/>
     </row>
     <row r="106" ht="15" customHeight="1" s="9">
       <c r="A106" s="11" t="n">
@@ -10476,6 +10581,7 @@
           <t>Blademaster:14</t>
         </is>
       </c>
+      <c r="Z106" t="inlineStr"/>
     </row>
     <row r="107" ht="15" customHeight="1" s="9">
       <c r="A107" s="13" t="n">
@@ -10575,6 +10681,7 @@
           <t>Blademaster:14</t>
         </is>
       </c>
+      <c r="Z107" t="inlineStr"/>
     </row>
     <row r="108" ht="15" customHeight="1" s="9">
       <c r="A108" s="11" t="n">
@@ -10670,6 +10777,7 @@
           <t>Blademaster:15</t>
         </is>
       </c>
+      <c r="Z108" t="inlineStr"/>
     </row>
     <row r="109" ht="15" customHeight="1" s="9">
       <c r="A109" s="13" t="n">
@@ -10765,6 +10873,7 @@
           <t>Blademaster:15</t>
         </is>
       </c>
+      <c r="Z109" t="inlineStr"/>
     </row>
     <row r="110" ht="15" customHeight="1" s="9">
       <c r="A110" s="11" t="n">
@@ -10856,6 +10965,7 @@
           <t>Blademaster:16</t>
         </is>
       </c>
+      <c r="Z110" t="inlineStr"/>
     </row>
     <row r="111" ht="15" customHeight="1" s="9">
       <c r="A111" s="13" t="n">
@@ -10955,6 +11065,7 @@
           <t>Blademaster:16</t>
         </is>
       </c>
+      <c r="Z111" t="inlineStr"/>
     </row>
     <row r="112" ht="15" customHeight="1" s="9">
       <c r="A112" s="11" t="n">
@@ -11052,6 +11163,7 @@
           <t>Blademaster:17</t>
         </is>
       </c>
+      <c r="Z112" t="inlineStr"/>
     </row>
     <row r="113" ht="15" customHeight="1" s="9">
       <c r="A113" s="13" t="n">
@@ -11143,6 +11255,7 @@
           <t>Blademaster:17</t>
         </is>
       </c>
+      <c r="Z113" t="inlineStr"/>
     </row>
     <row r="114" ht="15" customHeight="1" s="9">
       <c r="A114" s="11" t="n">
@@ -11234,6 +11347,7 @@
           <t>Blademaster:18</t>
         </is>
       </c>
+      <c r="Z114" t="inlineStr"/>
     </row>
     <row r="115" ht="15" customHeight="1" s="9">
       <c r="A115" s="13" t="n">
@@ -11325,6 +11439,7 @@
           <t>Blademaster:18</t>
         </is>
       </c>
+      <c r="Z115" t="inlineStr"/>
     </row>
     <row r="116" ht="15" customHeight="1" s="9">
       <c r="A116" s="11" t="n">
@@ -11420,6 +11535,7 @@
           <t>Blademaster:19</t>
         </is>
       </c>
+      <c r="Z116" t="inlineStr"/>
     </row>
     <row r="117" ht="15" customHeight="1" s="9">
       <c r="A117" s="13" t="n">
@@ -11511,6 +11627,7 @@
           <t>Blademaster:19</t>
         </is>
       </c>
+      <c r="Z117" t="inlineStr"/>
     </row>
     <row r="118" ht="15" customHeight="1" s="9">
       <c r="A118" s="11" t="n">
@@ -11606,6 +11723,7 @@
           <t>Blademaster:20</t>
         </is>
       </c>
+      <c r="Z118" t="inlineStr"/>
     </row>
     <row r="119" ht="15" customHeight="1" s="9">
       <c r="A119" s="13" t="n">
@@ -11701,6 +11819,7 @@
           <t>Blademaster:20</t>
         </is>
       </c>
+      <c r="Z119" t="inlineStr"/>
     </row>
     <row r="120" ht="15" customHeight="1" s="9">
       <c r="A120" s="11" t="n">
@@ -11796,6 +11915,7 @@
           <t>Blademaster:20</t>
         </is>
       </c>
+      <c r="Z120" t="inlineStr"/>
     </row>
     <row r="121" ht="15" customHeight="1" s="9">
       <c r="A121" s="13" t="n">
@@ -11891,6 +12011,7 @@
           <t>Lightmender:1</t>
         </is>
       </c>
+      <c r="Z121" t="inlineStr"/>
     </row>
     <row r="122" ht="15" customHeight="1" s="9">
       <c r="A122" s="11" t="n">
@@ -11986,6 +12107,11 @@
           <t>Lightmender:1</t>
         </is>
       </c>
+      <c r="Z122" t="inlineStr">
+        <is>
+          <t>You feel stronger by a blessing from the gods.</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="15" customHeight="1" s="9">
       <c r="A123" s="13" t="n">
@@ -12081,6 +12207,7 @@
           <t>Lightmender:2</t>
         </is>
       </c>
+      <c r="Z123" t="inlineStr"/>
     </row>
     <row r="124" ht="15" customHeight="1" s="9">
       <c r="A124" s="11" t="n">
@@ -12176,6 +12303,7 @@
           <t>Lightmender:2</t>
         </is>
       </c>
+      <c r="Z124" t="inlineStr"/>
     </row>
     <row r="125" ht="15" customHeight="1" s="9">
       <c r="A125" s="13" t="n">
@@ -12273,6 +12401,7 @@
           <t>Lightmender:3</t>
         </is>
       </c>
+      <c r="Z125" t="inlineStr"/>
     </row>
     <row r="126" ht="15" customHeight="1" s="9">
       <c r="A126" s="11" t="n">
@@ -12364,6 +12493,7 @@
           <t>Lightmender:3</t>
         </is>
       </c>
+      <c r="Z126" t="inlineStr"/>
     </row>
     <row r="127" ht="15" customHeight="1" s="9">
       <c r="A127" s="13" t="n">
@@ -12459,6 +12589,7 @@
           <t>Lightmender:4</t>
         </is>
       </c>
+      <c r="Z127" t="inlineStr"/>
     </row>
     <row r="128" ht="15" customHeight="1" s="9">
       <c r="A128" s="11" t="n">
@@ -12550,6 +12681,7 @@
           <t>Lightmender:4</t>
         </is>
       </c>
+      <c r="Z128" t="inlineStr"/>
     </row>
     <row r="129" ht="15" customHeight="1" s="9">
       <c r="A129" s="13" t="n">
@@ -12645,6 +12777,7 @@
           <t>Lightmender:5</t>
         </is>
       </c>
+      <c r="Z129" t="inlineStr"/>
     </row>
     <row r="130" ht="15" customHeight="1" s="9">
       <c r="A130" s="11" t="n">
@@ -12740,6 +12873,7 @@
           <t>Lightmender:5</t>
         </is>
       </c>
+      <c r="Z130" t="inlineStr"/>
     </row>
     <row r="131" ht="15" customHeight="1" s="9">
       <c r="A131" s="13" t="n">
@@ -12835,6 +12969,7 @@
           <t>Lightmender:6</t>
         </is>
       </c>
+      <c r="Z131" t="inlineStr"/>
     </row>
     <row r="132" ht="15" customHeight="1" s="9">
       <c r="A132" s="11" t="n">
@@ -12930,6 +13065,7 @@
           <t>Lightmender:6</t>
         </is>
       </c>
+      <c r="Z132" t="inlineStr"/>
     </row>
     <row r="133" ht="15" customHeight="1" s="9">
       <c r="A133" s="13" t="n">
@@ -13025,6 +13161,7 @@
           <t>Lightmender:7</t>
         </is>
       </c>
+      <c r="Z133" t="inlineStr"/>
     </row>
     <row r="134" ht="23.85" customHeight="1" s="9">
       <c r="A134" s="11" t="n">
@@ -13116,6 +13253,7 @@
           <t>Lightmender:1</t>
         </is>
       </c>
+      <c r="Z134" t="inlineStr"/>
     </row>
     <row r="135" ht="15" customHeight="1" s="9">
       <c r="A135" s="13" t="n">
@@ -13207,6 +13345,7 @@
           <t>Lightmender:8</t>
         </is>
       </c>
+      <c r="Z135" t="inlineStr"/>
     </row>
     <row r="136" ht="15" customHeight="1" s="9">
       <c r="A136" s="11" t="n">
@@ -13298,6 +13437,7 @@
           <t>Lightmender:8</t>
         </is>
       </c>
+      <c r="Z136" t="inlineStr"/>
     </row>
     <row r="137" ht="15" customHeight="1" s="9">
       <c r="A137" s="13" t="n">
@@ -13395,6 +13535,7 @@
           <t>Lightmender:9</t>
         </is>
       </c>
+      <c r="Z137" t="inlineStr"/>
     </row>
     <row r="138" ht="15" customHeight="1" s="9">
       <c r="A138" s="11" t="n">
@@ -13490,6 +13631,7 @@
           <t>Lightmender:9</t>
         </is>
       </c>
+      <c r="Z138" t="inlineStr"/>
     </row>
     <row r="139" ht="15" customHeight="1" s="9">
       <c r="A139" s="13" t="n">
@@ -13585,6 +13727,7 @@
           <t>Lightmender:10</t>
         </is>
       </c>
+      <c r="Z139" t="inlineStr"/>
     </row>
     <row r="140" ht="15" customHeight="1" s="9">
       <c r="A140" s="11" t="n">
@@ -13680,6 +13823,7 @@
           <t>Lightmender:10</t>
         </is>
       </c>
+      <c r="Z140" t="inlineStr"/>
     </row>
     <row r="141" ht="15" customHeight="1" s="9">
       <c r="A141" s="13" t="n">
@@ -13771,6 +13915,7 @@
           <t>Lightmender:11</t>
         </is>
       </c>
+      <c r="Z141" t="inlineStr"/>
     </row>
     <row r="142" ht="15" customHeight="1" s="9">
       <c r="A142" s="11" t="n">
@@ -13862,6 +14007,7 @@
           <t>Lightmender:11</t>
         </is>
       </c>
+      <c r="Z142" t="inlineStr"/>
     </row>
     <row r="143" ht="15" customHeight="1" s="9">
       <c r="A143" s="13" t="n">
@@ -13957,6 +14103,7 @@
           <t>Lightmender:12</t>
         </is>
       </c>
+      <c r="Z143" t="inlineStr"/>
     </row>
     <row r="144" ht="15" customHeight="1" s="9">
       <c r="A144" s="11" t="n">
@@ -14052,6 +14199,7 @@
           <t>Lightmender:12</t>
         </is>
       </c>
+      <c r="Z144" t="inlineStr"/>
     </row>
     <row r="145" ht="15" customHeight="1" s="9">
       <c r="A145" s="13" t="n">
@@ -14149,6 +14297,7 @@
           <t>Lightmender:13</t>
         </is>
       </c>
+      <c r="Z145" t="inlineStr"/>
     </row>
     <row r="146" ht="15" customHeight="1" s="9">
       <c r="A146" s="11" t="n">
@@ -14244,6 +14393,7 @@
           <t>Lightmender:13</t>
         </is>
       </c>
+      <c r="Z146" t="inlineStr"/>
     </row>
     <row r="147" ht="15" customHeight="1" s="9">
       <c r="A147" s="13" t="n">
@@ -14339,6 +14489,7 @@
           <t>Lightmender:14</t>
         </is>
       </c>
+      <c r="Z147" t="inlineStr"/>
     </row>
     <row r="148" ht="15" customHeight="1" s="9">
       <c r="A148" s="11" t="n">
@@ -14434,6 +14585,7 @@
           <t>Lightmender:14</t>
         </is>
       </c>
+      <c r="Z148" t="inlineStr"/>
     </row>
     <row r="149" ht="15" customHeight="1" s="9">
       <c r="A149" s="13" t="n">
@@ -14529,6 +14681,7 @@
           <t>Lightmender:15</t>
         </is>
       </c>
+      <c r="Z149" t="inlineStr"/>
     </row>
     <row r="150" ht="15" customHeight="1" s="9">
       <c r="A150" s="11" t="n">
@@ -14626,6 +14779,7 @@
           <t>Lightmender:15</t>
         </is>
       </c>
+      <c r="Z150" t="inlineStr"/>
     </row>
     <row r="151" ht="23.85" customHeight="1" s="9">
       <c r="A151" s="13" t="n">
@@ -14721,6 +14875,7 @@
           <t>Lightmender:16</t>
         </is>
       </c>
+      <c r="Z151" t="inlineStr"/>
     </row>
     <row r="152" ht="15" customHeight="1" s="9">
       <c r="A152" s="11" t="n">
@@ -14818,6 +14973,7 @@
           <t>Lightmender:17</t>
         </is>
       </c>
+      <c r="Z152" t="inlineStr"/>
     </row>
     <row r="153" ht="15" customHeight="1" s="9">
       <c r="A153" s="13" t="n">
@@ -14909,6 +15065,7 @@
           <t>Lightmender:17</t>
         </is>
       </c>
+      <c r="Z153" t="inlineStr"/>
     </row>
     <row r="154" ht="15" customHeight="1" s="9">
       <c r="A154" s="11" t="n">
@@ -15004,6 +15161,7 @@
           <t>Lightmender:18</t>
         </is>
       </c>
+      <c r="Z154" t="inlineStr"/>
     </row>
     <row r="155" ht="15" customHeight="1" s="9">
       <c r="A155" s="13" t="n">
@@ -15099,6 +15257,7 @@
           <t>Lightmender:18</t>
         </is>
       </c>
+      <c r="Z155" t="inlineStr"/>
     </row>
     <row r="156" ht="15" customHeight="1" s="9">
       <c r="A156" s="11" t="n">
@@ -15190,6 +15349,7 @@
           <t>Lightmender:19</t>
         </is>
       </c>
+      <c r="Z156" t="inlineStr"/>
     </row>
     <row r="157" ht="15" customHeight="1" s="9">
       <c r="A157" s="13" t="n">
@@ -15285,6 +15445,7 @@
           <t>Lightmender:19</t>
         </is>
       </c>
+      <c r="Z157" t="inlineStr"/>
     </row>
     <row r="158" ht="15" customHeight="1" s="9">
       <c r="A158" s="11" t="n">
@@ -15380,6 +15541,7 @@
           <t>Lightmender:20</t>
         </is>
       </c>
+      <c r="Z158" t="inlineStr"/>
     </row>
     <row r="159" ht="15" customHeight="1" s="9">
       <c r="A159" s="13" t="n">
@@ -15475,6 +15637,7 @@
           <t>Lightmender:20</t>
         </is>
       </c>
+      <c r="Z159" t="inlineStr"/>
     </row>
     <row r="160" ht="15" customHeight="1" s="9">
       <c r="A160" s="11" t="n">
@@ -15570,6 +15733,7 @@
           <t>Lightmender:20</t>
         </is>
       </c>
+      <c r="Z160" t="inlineStr"/>
     </row>
     <row r="161" ht="15" customHeight="1" s="9">
       <c r="A161" s="13" t="n">
@@ -15665,6 +15829,7 @@
           <t>Spiritcaller:1</t>
         </is>
       </c>
+      <c r="Z161" t="inlineStr"/>
     </row>
     <row r="162" ht="15" customHeight="1" s="9">
       <c r="A162" s="11" t="n">
@@ -15760,6 +15925,7 @@
           <t>Spiritcaller:1</t>
         </is>
       </c>
+      <c r="Z162" t="inlineStr"/>
     </row>
     <row r="163" ht="15" customHeight="1" s="9">
       <c r="A163" s="13" t="n">
@@ -15851,6 +16017,7 @@
           <t>Spiritcaller:2</t>
         </is>
       </c>
+      <c r="Z163" t="inlineStr"/>
     </row>
     <row r="164" ht="15" customHeight="1" s="9">
       <c r="A164" s="11" t="n">
@@ -15946,6 +16113,7 @@
           <t>Spiritcaller:2</t>
         </is>
       </c>
+      <c r="Z164" t="inlineStr"/>
     </row>
     <row r="165" ht="15" customHeight="1" s="9">
       <c r="A165" s="13" t="n">
@@ -16041,6 +16209,7 @@
           <t>Spiritcaller:3</t>
         </is>
       </c>
+      <c r="Z165" t="inlineStr"/>
     </row>
     <row r="166" ht="15" customHeight="1" s="9">
       <c r="A166" s="11" t="n">
@@ -16142,6 +16311,7 @@
           <t>Spiritcaller:3</t>
         </is>
       </c>
+      <c r="Z166" t="inlineStr"/>
     </row>
     <row r="167" ht="15" customHeight="1" s="9">
       <c r="A167" s="13" t="n">
@@ -16233,6 +16403,7 @@
           <t>Spiritcaller:4</t>
         </is>
       </c>
+      <c r="Z167" t="inlineStr"/>
     </row>
     <row r="168" ht="15" customHeight="1" s="9">
       <c r="A168" s="11" t="n">
@@ -16328,6 +16499,7 @@
           <t>Spiritcaller:4</t>
         </is>
       </c>
+      <c r="Z168" t="inlineStr"/>
     </row>
     <row r="169" ht="23.85" customHeight="1" s="9">
       <c r="A169" s="13" t="n">
@@ -16419,6 +16591,7 @@
           <t>Spiritcaller:5</t>
         </is>
       </c>
+      <c r="Z169" t="inlineStr"/>
     </row>
     <row r="170" ht="15" customHeight="1" s="9">
       <c r="A170" s="11" t="n">
@@ -16516,6 +16689,7 @@
           <t>Spiritcaller:5</t>
         </is>
       </c>
+      <c r="Z170" t="inlineStr"/>
     </row>
     <row r="171" ht="15" customHeight="1" s="9">
       <c r="A171" s="13" t="n">
@@ -16611,6 +16785,7 @@
           <t>Spiritcaller:6</t>
         </is>
       </c>
+      <c r="Z171" t="inlineStr"/>
     </row>
     <row r="172" ht="23.85" customHeight="1" s="9">
       <c r="A172" s="11" t="n">
@@ -16706,6 +16881,7 @@
           <t>Spiritcaller:6</t>
         </is>
       </c>
+      <c r="Z172" t="inlineStr"/>
     </row>
     <row r="173" ht="15" customHeight="1" s="9">
       <c r="A173" s="13" t="n">
@@ -16801,6 +16977,7 @@
           <t>Spiritcaller:7</t>
         </is>
       </c>
+      <c r="Z173" t="inlineStr"/>
     </row>
     <row r="174" ht="15" customHeight="1" s="9">
       <c r="A174" s="11" t="n">
@@ -16896,6 +17073,7 @@
           <t>Spiritcaller:7</t>
         </is>
       </c>
+      <c r="Z174" t="inlineStr"/>
     </row>
     <row r="175" ht="15" customHeight="1" s="9">
       <c r="A175" s="13" t="n">
@@ -16991,6 +17169,7 @@
           <t>Spiritcaller:8</t>
         </is>
       </c>
+      <c r="Z175" t="inlineStr"/>
     </row>
     <row r="176" ht="15" customHeight="1" s="9">
       <c r="A176" s="11" t="n">
@@ -17082,6 +17261,7 @@
           <t>Spiritcaller:8</t>
         </is>
       </c>
+      <c r="Z176" t="inlineStr"/>
     </row>
     <row r="177" ht="15" customHeight="1" s="9">
       <c r="A177" s="13" t="n">
@@ -17177,6 +17357,7 @@
           <t>Spiritcaller:9</t>
         </is>
       </c>
+      <c r="Z177" t="inlineStr"/>
     </row>
     <row r="178" ht="15" customHeight="1" s="9">
       <c r="A178" s="11" t="n">
@@ -17268,6 +17449,7 @@
           <t>Spiritcaller:9</t>
         </is>
       </c>
+      <c r="Z178" t="inlineStr"/>
     </row>
     <row r="179" ht="15" customHeight="1" s="9">
       <c r="A179" s="13" t="n">
@@ -17363,6 +17545,7 @@
           <t>Spiritcaller:10</t>
         </is>
       </c>
+      <c r="Z179" t="inlineStr"/>
     </row>
     <row r="180" ht="15" customHeight="1" s="9">
       <c r="A180" s="11" t="n">
@@ -17454,6 +17637,7 @@
           <t>Spiritcaller:10</t>
         </is>
       </c>
+      <c r="Z180" t="inlineStr"/>
     </row>
     <row r="181" ht="15" customHeight="1" s="9">
       <c r="A181" s="13" t="n">
@@ -17551,6 +17735,7 @@
           <t>Spiritcaller:11</t>
         </is>
       </c>
+      <c r="Z181" t="inlineStr"/>
     </row>
     <row r="182" ht="15" customHeight="1" s="9">
       <c r="A182" s="11" t="n">
@@ -17646,6 +17831,7 @@
           <t>Spiritcaller:11</t>
         </is>
       </c>
+      <c r="Z182" t="inlineStr"/>
     </row>
     <row r="183" ht="15" customHeight="1" s="9">
       <c r="A183" s="13" t="n">
@@ -17743,6 +17929,7 @@
           <t>Spiritcaller:12</t>
         </is>
       </c>
+      <c r="Z183" t="inlineStr"/>
     </row>
     <row r="184" ht="15" customHeight="1" s="9">
       <c r="A184" s="11" t="n">
@@ -17840,6 +18027,7 @@
           <t>Spiritcaller:12</t>
         </is>
       </c>
+      <c r="Z184" t="inlineStr"/>
     </row>
     <row r="185" ht="15" customHeight="1" s="9">
       <c r="A185" s="13" t="n">
@@ -17935,6 +18123,7 @@
           <t>Spiritcaller:13</t>
         </is>
       </c>
+      <c r="Z185" t="inlineStr"/>
     </row>
     <row r="186" ht="15" customHeight="1" s="9">
       <c r="A186" s="11" t="n">
@@ -18030,6 +18219,7 @@
           <t>Spiritcaller:13</t>
         </is>
       </c>
+      <c r="Z186" t="inlineStr"/>
     </row>
     <row r="187" ht="15" customHeight="1" s="9">
       <c r="A187" s="13" t="n">
@@ -18125,6 +18315,7 @@
           <t>Spiritcaller:14</t>
         </is>
       </c>
+      <c r="Z187" t="inlineStr"/>
     </row>
     <row r="188" ht="15" customHeight="1" s="9">
       <c r="A188" s="11" t="n">
@@ -18222,6 +18413,7 @@
           <t>Spiritcaller:14</t>
         </is>
       </c>
+      <c r="Z188" t="inlineStr"/>
     </row>
     <row r="189" ht="23.85" customHeight="1" s="9">
       <c r="A189" s="13" t="n">
@@ -18317,6 +18509,7 @@
           <t>Spiritcaller:15</t>
         </is>
       </c>
+      <c r="Z189" t="inlineStr"/>
     </row>
     <row r="190" ht="15" customHeight="1" s="9">
       <c r="A190" s="11" t="n">
@@ -18412,6 +18605,7 @@
           <t>Spiritcaller:15</t>
         </is>
       </c>
+      <c r="Z190" t="inlineStr"/>
     </row>
     <row r="191" ht="15" customHeight="1" s="9">
       <c r="A191" s="13" t="n">
@@ -18509,6 +18703,7 @@
           <t>Spiritcaller:16</t>
         </is>
       </c>
+      <c r="Z191" t="inlineStr"/>
     </row>
     <row r="192" ht="15" customHeight="1" s="9">
       <c r="A192" s="11" t="n">
@@ -18604,6 +18799,7 @@
           <t>Spiritcaller:16</t>
         </is>
       </c>
+      <c r="Z192" t="inlineStr"/>
     </row>
     <row r="193" ht="23.85" customHeight="1" s="9">
       <c r="A193" s="13" t="n">
@@ -18695,6 +18891,7 @@
           <t>Spiritcaller:17</t>
         </is>
       </c>
+      <c r="Z193" t="inlineStr"/>
     </row>
     <row r="194" ht="15" customHeight="1" s="9">
       <c r="A194" s="11" t="n">
@@ -18790,6 +18987,7 @@
           <t>Spiritcaller:17</t>
         </is>
       </c>
+      <c r="Z194" t="inlineStr"/>
     </row>
     <row r="195" ht="15" customHeight="1" s="9">
       <c r="A195" s="13" t="n">
@@ -18885,6 +19083,7 @@
           <t>Spiritcaller:18</t>
         </is>
       </c>
+      <c r="Z195" t="inlineStr"/>
     </row>
     <row r="196" ht="15" customHeight="1" s="9">
       <c r="A196" s="11" t="n">
@@ -18980,6 +19179,7 @@
           <t>Spiritcaller:18</t>
         </is>
       </c>
+      <c r="Z196" t="inlineStr"/>
     </row>
     <row r="197" ht="23.85" customHeight="1" s="9">
       <c r="A197" s="13" t="n">
@@ -19077,6 +19277,7 @@
           <t>Spiritcaller:19</t>
         </is>
       </c>
+      <c r="Z197" t="inlineStr"/>
     </row>
     <row r="198" ht="15" customHeight="1" s="9">
       <c r="A198" s="11" t="n">
@@ -19168,6 +19369,7 @@
           <t>Spiritcaller:19</t>
         </is>
       </c>
+      <c r="Z198" t="inlineStr"/>
     </row>
     <row r="199" ht="15" customHeight="1" s="9">
       <c r="A199" s="13" t="n">
@@ -19263,6 +19465,7 @@
           <t>Spiritcaller:20</t>
         </is>
       </c>
+      <c r="Z199" t="inlineStr"/>
     </row>
     <row r="200" ht="15" customHeight="1" s="9">
       <c r="A200" s="11" t="n">
@@ -19358,6 +19561,7 @@
           <t>Spiritcaller:20</t>
         </is>
       </c>
+      <c r="Z200" t="inlineStr"/>
     </row>
     <row r="201" ht="15" customHeight="1" s="9">
       <c r="A201" s="13" t="n">
@@ -19455,6 +19659,7 @@
           <t>Spiritcaller:20</t>
         </is>
       </c>
+      <c r="Z201" t="inlineStr"/>
     </row>
     <row r="202" ht="15" customHeight="1" s="9">
       <c r="A202" s="11" t="n">
@@ -19552,6 +19757,7 @@
           <t>Wildspeaker:1</t>
         </is>
       </c>
+      <c r="Z202" t="inlineStr"/>
     </row>
     <row r="203" ht="15" customHeight="1" s="9">
       <c r="A203" s="13" t="n">
@@ -19651,6 +19857,7 @@
           <t>Wildspeaker:1</t>
         </is>
       </c>
+      <c r="Z203" t="inlineStr"/>
     </row>
     <row r="204" ht="15" customHeight="1" s="9">
       <c r="A204" s="11" t="n">
@@ -19746,6 +19953,7 @@
           <t>Wildspeaker:2</t>
         </is>
       </c>
+      <c r="Z204" t="inlineStr"/>
     </row>
     <row r="205" ht="15" customHeight="1" s="9">
       <c r="A205" s="13" t="n">
@@ -19837,6 +20045,7 @@
           <t>Wildspeaker:2</t>
         </is>
       </c>
+      <c r="Z205" t="inlineStr"/>
     </row>
     <row r="206" ht="15" customHeight="1" s="9">
       <c r="A206" s="11" t="n">
@@ -19934,6 +20143,7 @@
           <t>Wildspeaker:3</t>
         </is>
       </c>
+      <c r="Z206" t="inlineStr"/>
     </row>
     <row r="207" ht="15" customHeight="1" s="9">
       <c r="A207" s="13" t="n">
@@ -20025,6 +20235,7 @@
           <t>Wildspeaker:3</t>
         </is>
       </c>
+      <c r="Z207" t="inlineStr"/>
     </row>
     <row r="208" ht="15" customHeight="1" s="9">
       <c r="A208" s="11" t="n">
@@ -20120,6 +20331,7 @@
           <t>Wildspeaker:4</t>
         </is>
       </c>
+      <c r="Z208" t="inlineStr"/>
     </row>
     <row r="209" ht="15" customHeight="1" s="9">
       <c r="A209" s="13" t="n">
@@ -20215,6 +20427,7 @@
           <t>Wildspeaker:4</t>
         </is>
       </c>
+      <c r="Z209" t="inlineStr"/>
     </row>
     <row r="210" ht="15" customHeight="1" s="9">
       <c r="A210" s="11" t="n">
@@ -20312,6 +20525,7 @@
           <t>Wildspeaker:5</t>
         </is>
       </c>
+      <c r="Z210" t="inlineStr"/>
     </row>
     <row r="211" ht="15" customHeight="1" s="9">
       <c r="A211" s="13" t="n">
@@ -20403,6 +20617,7 @@
           <t>Wildspeaker:5</t>
         </is>
       </c>
+      <c r="Z211" t="inlineStr"/>
     </row>
     <row r="212" ht="15" customHeight="1" s="9">
       <c r="A212" s="11" t="n">
@@ -20494,6 +20709,7 @@
           <t>Wildspeaker:6</t>
         </is>
       </c>
+      <c r="Z212" t="inlineStr"/>
     </row>
     <row r="213" ht="15" customHeight="1" s="9">
       <c r="A213" s="13" t="n">
@@ -20585,6 +20801,7 @@
           <t>Wildspeaker:6</t>
         </is>
       </c>
+      <c r="Z213" t="inlineStr"/>
     </row>
     <row r="214" ht="15" customHeight="1" s="9">
       <c r="A214" s="11" t="n">
@@ -20682,6 +20899,7 @@
           <t>Wildspeaker:7</t>
         </is>
       </c>
+      <c r="Z214" t="inlineStr"/>
     </row>
     <row r="215" ht="15" customHeight="1" s="9">
       <c r="A215" s="13" t="n">
@@ -20773,6 +20991,7 @@
           <t>Wildspeaker:7</t>
         </is>
       </c>
+      <c r="Z215" t="inlineStr"/>
     </row>
     <row r="216" ht="23.85" customHeight="1" s="9">
       <c r="A216" s="11" t="n">
@@ -20868,6 +21087,7 @@
           <t>Wildspeaker:8</t>
         </is>
       </c>
+      <c r="Z216" t="inlineStr"/>
     </row>
     <row r="217" ht="15" customHeight="1" s="9">
       <c r="A217" s="13" t="n">
@@ -20959,6 +21179,7 @@
           <t>Wildspeaker:8</t>
         </is>
       </c>
+      <c r="Z217" t="inlineStr"/>
     </row>
     <row r="218" ht="23.85" customHeight="1" s="9">
       <c r="A218" s="11" t="n">
@@ -21054,6 +21275,7 @@
           <t>Wildspeaker:9</t>
         </is>
       </c>
+      <c r="Z218" t="inlineStr"/>
     </row>
     <row r="219" ht="15" customHeight="1" s="9">
       <c r="A219" s="13" t="n">
@@ -21151,6 +21373,7 @@
           <t>Wildspeaker:9</t>
         </is>
       </c>
+      <c r="Z219" t="inlineStr"/>
     </row>
     <row r="220" ht="15" customHeight="1" s="9">
       <c r="A220" s="11" t="n">
@@ -21246,6 +21469,7 @@
           <t>Wildspeaker:10</t>
         </is>
       </c>
+      <c r="Z220" t="inlineStr"/>
     </row>
     <row r="221" ht="15" customHeight="1" s="9">
       <c r="A221" s="13" t="n">
@@ -21337,6 +21561,7 @@
           <t>Wildspeaker:10</t>
         </is>
       </c>
+      <c r="Z221" t="inlineStr"/>
     </row>
     <row r="222" ht="15" customHeight="1" s="9">
       <c r="A222" s="11" t="n">
@@ -21432,6 +21657,7 @@
           <t>Wildspeaker:11</t>
         </is>
       </c>
+      <c r="Z222" t="inlineStr"/>
     </row>
     <row r="223" ht="15" customHeight="1" s="9">
       <c r="A223" s="13" t="n">
@@ -21527,6 +21753,7 @@
           <t>Wildspeaker:11</t>
         </is>
       </c>
+      <c r="Z223" t="inlineStr"/>
     </row>
     <row r="224" ht="23.85" customHeight="1" s="9">
       <c r="A224" s="11" t="n">
@@ -21622,6 +21849,7 @@
           <t>Wildspeaker:12</t>
         </is>
       </c>
+      <c r="Z224" t="inlineStr"/>
     </row>
     <row r="225" ht="15" customHeight="1" s="9">
       <c r="A225" s="13" t="n">
@@ -21713,6 +21941,7 @@
           <t>Wildspeaker:12</t>
         </is>
       </c>
+      <c r="Z225" t="inlineStr"/>
     </row>
     <row r="226" ht="15" customHeight="1" s="9">
       <c r="A226" s="11" t="n">
@@ -21810,6 +22039,7 @@
           <t>Wildspeaker:13</t>
         </is>
       </c>
+      <c r="Z226" t="inlineStr"/>
     </row>
     <row r="227" ht="15" customHeight="1" s="9">
       <c r="A227" s="13" t="n">
@@ -21905,6 +22135,7 @@
           <t>Wildspeaker:13</t>
         </is>
       </c>
+      <c r="Z227" t="inlineStr"/>
     </row>
     <row r="228" ht="15" customHeight="1" s="9">
       <c r="A228" s="11" t="n">
@@ -22002,6 +22233,7 @@
           <t>Wildspeaker:14</t>
         </is>
       </c>
+      <c r="Z228" t="inlineStr"/>
     </row>
     <row r="229" ht="23.85" customHeight="1" s="9">
       <c r="A229" s="13" t="n">
@@ -22103,6 +22335,7 @@
           <t>Wildspeaker:14</t>
         </is>
       </c>
+      <c r="Z229" t="inlineStr"/>
     </row>
     <row r="230" ht="15" customHeight="1" s="9">
       <c r="A230" s="11" t="n">
@@ -22198,6 +22431,7 @@
           <t>Wildspeaker:15</t>
         </is>
       </c>
+      <c r="Z230" t="inlineStr"/>
     </row>
     <row r="231" ht="15" customHeight="1" s="9">
       <c r="A231" s="13" t="n">
@@ -22293,6 +22527,7 @@
           <t>Wildspeaker:15</t>
         </is>
       </c>
+      <c r="Z231" t="inlineStr"/>
     </row>
     <row r="232" ht="15" customHeight="1" s="9">
       <c r="A232" s="11" t="n">
@@ -22388,6 +22623,7 @@
           <t>Wildspeaker:16</t>
         </is>
       </c>
+      <c r="Z232" t="inlineStr"/>
     </row>
     <row r="233" ht="15" customHeight="1" s="9">
       <c r="A233" s="13" t="n">
@@ -22483,6 +22719,7 @@
           <t>Wildspeaker:16</t>
         </is>
       </c>
+      <c r="Z233" t="inlineStr"/>
     </row>
     <row r="234" ht="23.85" customHeight="1" s="9">
       <c r="A234" s="11" t="n">
@@ -22578,6 +22815,7 @@
           <t>Wildspeaker:17</t>
         </is>
       </c>
+      <c r="Z234" t="inlineStr"/>
     </row>
     <row r="235" ht="15" customHeight="1" s="9">
       <c r="A235" s="13" t="n">
@@ -22673,6 +22911,7 @@
           <t>Wildspeaker:17</t>
         </is>
       </c>
+      <c r="Z235" t="inlineStr"/>
     </row>
     <row r="236" ht="15" customHeight="1" s="9">
       <c r="A236" s="11" t="n">
@@ -22770,6 +23009,7 @@
           <t>Wildspeaker:18</t>
         </is>
       </c>
+      <c r="Z236" t="inlineStr"/>
     </row>
     <row r="237" ht="15" customHeight="1" s="9">
       <c r="A237" s="13" t="n">
@@ -22861,6 +23101,7 @@
           <t>Wildspeaker:18</t>
         </is>
       </c>
+      <c r="Z237" t="inlineStr"/>
     </row>
     <row r="238" ht="15" customHeight="1" s="9">
       <c r="A238" s="11" t="n">
@@ -22952,6 +23193,7 @@
           <t>Wildspeaker:19</t>
         </is>
       </c>
+      <c r="Z238" t="inlineStr"/>
     </row>
     <row r="239" ht="15" customHeight="1" s="9">
       <c r="A239" s="13" t="n">
@@ -23144,6 +23386,7 @@
           <t>Wildspeaker:20</t>
         </is>
       </c>
+      <c r="Z240" t="inlineStr"/>
     </row>
     <row r="241" ht="15" customHeight="1" s="9">
       <c r="A241" s="13" t="n">
@@ -23239,6 +23482,7 @@
           <t>Wildspeaker:20</t>
         </is>
       </c>
+      <c r="Z241" t="inlineStr"/>
     </row>
     <row r="242" ht="15" customHeight="1" s="9">
       <c r="A242" s="11" t="n">
@@ -23334,6 +23578,7 @@
           <t>Wildspeaker:20</t>
         </is>
       </c>
+      <c r="Z242" t="inlineStr"/>
     </row>
     <row r="243" ht="15" customHeight="1" s="9">
       <c r="A243" s="13" t="n">
@@ -23425,6 +23670,7 @@
           <t>Zenblade:1</t>
         </is>
       </c>
+      <c r="Z243" t="inlineStr"/>
     </row>
     <row r="244" ht="15" customHeight="1" s="9">
       <c r="A244" s="11" t="n">
@@ -23516,6 +23762,7 @@
           <t>Zenblade:1</t>
         </is>
       </c>
+      <c r="Z244" t="inlineStr"/>
     </row>
     <row r="245" ht="15" customHeight="1" s="9">
       <c r="A245" s="13" t="n">
@@ -23607,6 +23854,7 @@
           <t>Zenblade:2</t>
         </is>
       </c>
+      <c r="Z245" t="inlineStr"/>
     </row>
     <row r="246" ht="15" customHeight="1" s="9">
       <c r="A246" s="11" t="n">
@@ -23702,6 +23950,7 @@
           <t>Zenblade:2</t>
         </is>
       </c>
+      <c r="Z246" t="inlineStr"/>
     </row>
     <row r="247" ht="15" customHeight="1" s="9">
       <c r="A247" s="13" t="n">
@@ -23793,6 +24042,7 @@
           <t>Zenblade:3</t>
         </is>
       </c>
+      <c r="Z247" t="inlineStr"/>
     </row>
     <row r="248" ht="15" customHeight="1" s="9">
       <c r="A248" s="11" t="n">
@@ -23890,6 +24140,7 @@
           <t>Zenblade:3</t>
         </is>
       </c>
+      <c r="Z248" t="inlineStr"/>
     </row>
     <row r="249" ht="15" customHeight="1" s="9">
       <c r="A249" s="13" t="n">
@@ -23987,6 +24238,7 @@
           <t>Zenblade:4</t>
         </is>
       </c>
+      <c r="Z249" t="inlineStr"/>
     </row>
     <row r="250" ht="15" customHeight="1" s="9">
       <c r="A250" s="11" t="n">
@@ -24082,6 +24334,7 @@
           <t>Zenblade:4</t>
         </is>
       </c>
+      <c r="Z250" t="inlineStr"/>
     </row>
     <row r="251" ht="15" customHeight="1" s="9">
       <c r="A251" s="13" t="n">
@@ -24179,6 +24432,7 @@
           <t>Zenblade:5</t>
         </is>
       </c>
+      <c r="Z251" t="inlineStr"/>
     </row>
     <row r="252" ht="15" customHeight="1" s="9">
       <c r="A252" s="11" t="n">
@@ -24274,6 +24528,7 @@
           <t>Zenblade:5</t>
         </is>
       </c>
+      <c r="Z252" t="inlineStr"/>
     </row>
     <row r="253" ht="15" customHeight="1" s="9">
       <c r="A253" s="13" t="n">
@@ -24369,6 +24624,7 @@
           <t>Zenblade:6</t>
         </is>
       </c>
+      <c r="Z253" t="inlineStr"/>
     </row>
     <row r="254" ht="15" customHeight="1" s="9">
       <c r="A254" s="11" t="n">
@@ -24460,6 +24716,7 @@
           <t>Zenblade:6</t>
         </is>
       </c>
+      <c r="Z254" t="inlineStr"/>
     </row>
     <row r="255" ht="15" customHeight="1" s="9">
       <c r="A255" s="13" t="n">
@@ -24551,6 +24808,7 @@
           <t>Zenblade:7</t>
         </is>
       </c>
+      <c r="Z255" t="inlineStr"/>
     </row>
     <row r="256" ht="15" customHeight="1" s="9">
       <c r="A256" s="11" t="n">
@@ -24642,6 +24900,7 @@
           <t>Zenblade:8</t>
         </is>
       </c>
+      <c r="Z256" t="inlineStr"/>
     </row>
     <row r="257" ht="15" customHeight="1" s="9">
       <c r="A257" s="13" t="n">
@@ -24733,6 +24992,7 @@
           <t>Zenblade:8</t>
         </is>
       </c>
+      <c r="Z257" t="inlineStr"/>
     </row>
     <row r="258" ht="15" customHeight="1" s="9">
       <c r="A258" s="11" t="n">
@@ -24828,6 +25088,7 @@
           <t>Zenblade:9</t>
         </is>
       </c>
+      <c r="Z258" t="inlineStr"/>
     </row>
     <row r="259" ht="15" customHeight="1" s="9">
       <c r="A259" s="13" t="n">
@@ -24919,6 +25180,7 @@
           <t>Zenblade:9</t>
         </is>
       </c>
+      <c r="Z259" t="inlineStr"/>
     </row>
     <row r="260" ht="15" customHeight="1" s="9">
       <c r="A260" s="11" t="n">
@@ -25012,6 +25274,7 @@
           <t>Zenblade:10</t>
         </is>
       </c>
+      <c r="Z260" t="inlineStr"/>
     </row>
     <row r="261" ht="15" customHeight="1" s="9">
       <c r="A261" s="13" t="n">
@@ -25103,6 +25366,7 @@
           <t>Zenblade:10</t>
         </is>
       </c>
+      <c r="Z261" t="inlineStr"/>
     </row>
     <row r="262" ht="15" customHeight="1" s="9">
       <c r="A262" s="11" t="n">
@@ -25198,6 +25462,7 @@
           <t>Zenblade:11</t>
         </is>
       </c>
+      <c r="Z262" t="inlineStr"/>
     </row>
     <row r="263" ht="15" customHeight="1" s="9">
       <c r="A263" s="13" t="n">
@@ -25293,6 +25558,7 @@
           <t>Zenblade:11</t>
         </is>
       </c>
+      <c r="Z263" t="inlineStr"/>
     </row>
     <row r="264" ht="15" customHeight="1" s="9">
       <c r="A264" s="11" t="n">
@@ -25384,6 +25650,7 @@
           <t>Zenblade:12</t>
         </is>
       </c>
+      <c r="Z264" t="inlineStr"/>
     </row>
     <row r="265" ht="15" customHeight="1" s="9">
       <c r="A265" s="13" t="n">
@@ -25475,6 +25742,7 @@
           <t>Zenblade:12</t>
         </is>
       </c>
+      <c r="Z265" t="inlineStr"/>
     </row>
     <row r="266" ht="15" customHeight="1" s="9">
       <c r="A266" s="11" t="n">
@@ -25566,6 +25834,7 @@
           <t>Zenblade:13</t>
         </is>
       </c>
+      <c r="Z266" t="inlineStr"/>
     </row>
     <row r="267" ht="15" customHeight="1" s="9">
       <c r="A267" s="13" t="n">
@@ -25657,6 +25926,7 @@
           <t>Zenblade:13</t>
         </is>
       </c>
+      <c r="Z267" t="inlineStr"/>
     </row>
     <row r="268" ht="15" customHeight="1" s="9">
       <c r="A268" s="11" t="n">
@@ -25752,6 +26022,7 @@
           <t>Zenblade:14</t>
         </is>
       </c>
+      <c r="Z268" t="inlineStr"/>
     </row>
     <row r="269" ht="15" customHeight="1" s="9">
       <c r="A269" s="13" t="n">
@@ -25843,6 +26114,7 @@
           <t>Zenblade:14</t>
         </is>
       </c>
+      <c r="Z269" t="inlineStr"/>
     </row>
     <row r="270" ht="15" customHeight="1" s="9">
       <c r="A270" s="11" t="n">
@@ -25934,6 +26206,7 @@
           <t>Zenblade:15</t>
         </is>
       </c>
+      <c r="Z270" t="inlineStr"/>
     </row>
     <row r="271" ht="15" customHeight="1" s="9">
       <c r="A271" s="13" t="n">
@@ -26025,6 +26298,7 @@
           <t>Zenblade:15</t>
         </is>
       </c>
+      <c r="Z271" t="inlineStr"/>
     </row>
     <row r="272" ht="15" customHeight="1" s="9">
       <c r="A272" s="11" t="n">
@@ -26116,6 +26390,7 @@
           <t>Zenblade:16</t>
         </is>
       </c>
+      <c r="Z272" t="inlineStr"/>
     </row>
     <row r="273" ht="15" customHeight="1" s="9">
       <c r="A273" s="13" t="n">
@@ -26211,6 +26486,7 @@
           <t>Zenblade:16</t>
         </is>
       </c>
+      <c r="Z273" t="inlineStr"/>
     </row>
     <row r="274" ht="15" customHeight="1" s="9">
       <c r="A274" s="11" t="n">
@@ -26302,6 +26578,7 @@
           <t>Zenblade:17</t>
         </is>
       </c>
+      <c r="Z274" t="inlineStr"/>
     </row>
     <row r="275" ht="15" customHeight="1" s="9">
       <c r="A275" s="13" t="n">
@@ -26393,6 +26670,7 @@
           <t>Zenblade:17</t>
         </is>
       </c>
+      <c r="Z275" t="inlineStr"/>
     </row>
     <row r="276" ht="15" customHeight="1" s="9">
       <c r="A276" s="11" t="n">
@@ -26488,6 +26766,7 @@
           <t>Zenblade:18</t>
         </is>
       </c>
+      <c r="Z276" t="inlineStr"/>
     </row>
     <row r="277" ht="15" customHeight="1" s="9">
       <c r="A277" s="13" t="n">
@@ -26579,6 +26858,7 @@
           <t>Zenblade:18</t>
         </is>
       </c>
+      <c r="Z277" t="inlineStr"/>
     </row>
     <row r="278" ht="15" customHeight="1" s="9">
       <c r="A278" s="11" t="n">
@@ -26674,6 +26954,7 @@
           <t>Zenblade:19</t>
         </is>
       </c>
+      <c r="Z278" t="inlineStr"/>
     </row>
     <row r="279" ht="15" customHeight="1" s="9">
       <c r="A279" s="13" t="n">
@@ -26864,6 +27145,7 @@
           <t>Zenblade:20</t>
         </is>
       </c>
+      <c r="Z280" t="inlineStr"/>
     </row>
     <row r="281" ht="15" customHeight="1" s="9">
       <c r="A281" s="13" t="n">
@@ -26959,6 +27241,7 @@
           <t>Zenblade:20</t>
         </is>
       </c>
+      <c r="Z281" t="inlineStr"/>
     </row>
     <row r="282" ht="15" customHeight="1" s="9">
       <c r="A282" s="11" t="n">
@@ -27054,6 +27337,7 @@
           <t>Zenblade:20</t>
         </is>
       </c>
+      <c r="Z282" t="inlineStr"/>
     </row>
     <row r="283" ht="15" customHeight="1" s="9">
       <c r="A283" s="13" t="n">
@@ -27145,6 +27429,7 @@
           <t>Woodstalker:1</t>
         </is>
       </c>
+      <c r="Z283" t="inlineStr"/>
     </row>
     <row r="284" ht="23.85" customHeight="1" s="9">
       <c r="A284" s="11" t="n">
@@ -27240,6 +27525,7 @@
           <t>Woodstalker:1</t>
         </is>
       </c>
+      <c r="Z284" t="inlineStr"/>
     </row>
     <row r="285" ht="15" customHeight="1" s="9">
       <c r="A285" s="13" t="n">
@@ -27335,6 +27621,7 @@
           <t>Woodstalker:2</t>
         </is>
       </c>
+      <c r="Z285" t="inlineStr"/>
     </row>
     <row r="286" ht="15" customHeight="1" s="9">
       <c r="A286" s="11" t="n">
@@ -27434,6 +27721,7 @@
           <t>Woodstalker:2</t>
         </is>
       </c>
+      <c r="Z286" t="inlineStr"/>
     </row>
     <row r="287" ht="23.85" customHeight="1" s="9">
       <c r="A287" s="13" t="n">
@@ -27529,6 +27817,7 @@
           <t>Shadowblade:3, Troubadour:3, Woodstalker:3</t>
         </is>
       </c>
+      <c r="Z287" t="inlineStr"/>
     </row>
     <row r="288" ht="15" customHeight="1" s="9">
       <c r="A288" s="11" t="n">
@@ -27620,6 +27909,7 @@
           <t>Woodstalker:3</t>
         </is>
       </c>
+      <c r="Z288" t="inlineStr"/>
     </row>
     <row r="289" ht="15" customHeight="1" s="9">
       <c r="A289" s="13" t="n">
@@ -27715,6 +28005,7 @@
           <t>Woodstalker:4</t>
         </is>
       </c>
+      <c r="Z289" t="inlineStr"/>
     </row>
     <row r="290" ht="15" customHeight="1" s="9">
       <c r="A290" s="11" t="n">
@@ -27812,6 +28103,7 @@
           <t>Woodstalker:4</t>
         </is>
       </c>
+      <c r="Z290" t="inlineStr"/>
     </row>
     <row r="291" ht="23.85" customHeight="1" s="9">
       <c r="A291" s="13" t="n">
@@ -27903,6 +28195,7 @@
           <t>Shadowblade:5, Troubadour:5, Woodstalker:5</t>
         </is>
       </c>
+      <c r="Z291" t="inlineStr"/>
     </row>
     <row r="292" ht="15" customHeight="1" s="9">
       <c r="A292" s="11" t="n">
@@ -27994,6 +28287,7 @@
           <t>Woodstalker:5</t>
         </is>
       </c>
+      <c r="Z292" t="inlineStr"/>
     </row>
     <row r="293" ht="23.85" customHeight="1" s="9">
       <c r="A293" s="13" t="n">
@@ -28091,6 +28385,7 @@
           <t>Woodstalker:6</t>
         </is>
       </c>
+      <c r="Z293" t="inlineStr"/>
     </row>
     <row r="294" ht="15" customHeight="1" s="9">
       <c r="A294" s="11" t="n">
@@ -28182,6 +28477,7 @@
           <t>Woodstalker:6</t>
         </is>
       </c>
+      <c r="Z294" t="inlineStr"/>
     </row>
     <row r="295" ht="23.85" customHeight="1" s="9">
       <c r="A295" s="13" t="n">
@@ -28277,6 +28573,7 @@
           <t>Shadowblade:7, Troubadour:7, Woodstalker:7</t>
         </is>
       </c>
+      <c r="Z295" t="inlineStr"/>
     </row>
     <row r="296" ht="15" customHeight="1" s="9">
       <c r="A296" s="11" t="n">
@@ -28372,6 +28669,7 @@
           <t>Woodstalker:7</t>
         </is>
       </c>
+      <c r="Z296" t="inlineStr"/>
     </row>
     <row r="297" ht="15" customHeight="1" s="9">
       <c r="A297" s="13" t="n">
@@ -28467,6 +28765,7 @@
           <t>Woodstalker:8</t>
         </is>
       </c>
+      <c r="Z297" t="inlineStr"/>
     </row>
     <row r="298" ht="15" customHeight="1" s="9">
       <c r="A298" s="11" t="n">
@@ -28558,6 +28857,7 @@
           <t>Woodstalker:8</t>
         </is>
       </c>
+      <c r="Z298" t="inlineStr"/>
     </row>
     <row r="299" ht="15" customHeight="1" s="9">
       <c r="A299" s="13" t="n">
@@ -28655,6 +28955,7 @@
           <t>Woodstalker:9</t>
         </is>
       </c>
+      <c r="Z299" t="inlineStr"/>
     </row>
     <row r="300" ht="15" customHeight="1" s="9">
       <c r="A300" s="11" t="n">
@@ -28746,6 +29047,7 @@
           <t>Woodstalker:9</t>
         </is>
       </c>
+      <c r="Z300" t="inlineStr"/>
     </row>
     <row r="301" ht="23.85" customHeight="1" s="9">
       <c r="A301" s="13" t="n">
@@ -28837,6 +29139,7 @@
           <t>Shadowblade:10, Troubadour:10, Woodstalker:10</t>
         </is>
       </c>
+      <c r="Z301" t="inlineStr"/>
     </row>
     <row r="302" ht="15" customHeight="1" s="9">
       <c r="A302" s="11" t="n">
@@ -28928,6 +29231,7 @@
           <t>Woodstalker:10</t>
         </is>
       </c>
+      <c r="Z302" t="inlineStr"/>
     </row>
     <row r="303" ht="15" customHeight="1" s="9">
       <c r="A303" s="13" t="n">
@@ -29019,6 +29323,7 @@
           <t>Woodstalker:11</t>
         </is>
       </c>
+      <c r="Z303" t="inlineStr"/>
     </row>
     <row r="304" ht="15" customHeight="1" s="9">
       <c r="A304" s="11" t="n">
@@ -29110,6 +29415,7 @@
           <t>Woodstalker:11</t>
         </is>
       </c>
+      <c r="Z304" t="inlineStr"/>
     </row>
     <row r="305" ht="15" customHeight="1" s="9">
       <c r="A305" s="13" t="n">
@@ -29205,6 +29511,7 @@
           <t>Woodstalker:12</t>
         </is>
       </c>
+      <c r="Z305" t="inlineStr"/>
     </row>
     <row r="306" ht="15" customHeight="1" s="9">
       <c r="A306" s="11" t="n">
@@ -29296,6 +29603,7 @@
           <t>Woodstalker:12</t>
         </is>
       </c>
+      <c r="Z306" t="inlineStr"/>
     </row>
     <row r="307" ht="15" customHeight="1" s="9">
       <c r="A307" s="13" t="n">
@@ -29391,6 +29699,7 @@
           <t>Woodstalker:13</t>
         </is>
       </c>
+      <c r="Z307" t="inlineStr"/>
     </row>
     <row r="308" ht="15" customHeight="1" s="9">
       <c r="A308" s="11" t="n">
@@ -29482,6 +29791,7 @@
           <t>Woodstalker:13</t>
         </is>
       </c>
+      <c r="Z308" t="inlineStr"/>
     </row>
     <row r="309" ht="23.85" customHeight="1" s="9">
       <c r="A309" s="13" t="n">
@@ -29573,6 +29883,7 @@
           <t>Shadowblade:14, Troubadour:14, Woodstalker:14</t>
         </is>
       </c>
+      <c r="Z309" t="inlineStr"/>
     </row>
     <row r="310" ht="15" customHeight="1" s="9">
       <c r="A310" s="11" t="n">
@@ -29664,6 +29975,7 @@
           <t>Woodstalker:14</t>
         </is>
       </c>
+      <c r="Z310" t="inlineStr"/>
     </row>
     <row r="311" ht="23.85" customHeight="1" s="9">
       <c r="A311" s="13" t="n">
@@ -29759,6 +30071,7 @@
           <t>Woodstalker:15</t>
         </is>
       </c>
+      <c r="Z311" t="inlineStr"/>
     </row>
     <row r="312" ht="15" customHeight="1" s="9">
       <c r="A312" s="11" t="n">
@@ -29850,6 +30163,7 @@
           <t>Woodstalker:15</t>
         </is>
       </c>
+      <c r="Z312" t="inlineStr"/>
     </row>
     <row r="313" ht="15" customHeight="1" s="9">
       <c r="A313" s="13" t="n">
@@ -29941,6 +30255,7 @@
           <t>Woodstalker:16</t>
         </is>
       </c>
+      <c r="Z313" t="inlineStr"/>
     </row>
     <row r="314" ht="15" customHeight="1" s="9">
       <c r="A314" s="11" t="n">
@@ -30036,6 +30351,7 @@
           <t>Woodstalker:16</t>
         </is>
       </c>
+      <c r="Z314" t="inlineStr"/>
     </row>
     <row r="315" ht="23.85" customHeight="1" s="9">
       <c r="A315" s="13" t="n">
@@ -30131,6 +30447,7 @@
           <t>Woodstalker:17</t>
         </is>
       </c>
+      <c r="Z315" t="inlineStr"/>
     </row>
     <row r="316" ht="15" customHeight="1" s="9">
       <c r="A316" s="11" t="n">
@@ -30226,6 +30543,7 @@
           <t>Woodstalker:17</t>
         </is>
       </c>
+      <c r="Z316" t="inlineStr"/>
     </row>
     <row r="317" ht="15" customHeight="1" s="9">
       <c r="A317" s="13" t="n">
@@ -30317,6 +30635,7 @@
           <t>Woodstalker:18</t>
         </is>
       </c>
+      <c r="Z317" t="inlineStr"/>
     </row>
     <row r="318" ht="23.85" customHeight="1" s="9">
       <c r="A318" s="11" t="n">
@@ -30416,6 +30735,7 @@
           <t>Woodstalker:18</t>
         </is>
       </c>
+      <c r="Z318" t="inlineStr"/>
     </row>
     <row r="319" ht="15" customHeight="1" s="9">
       <c r="A319" s="13" t="n">
@@ -30511,6 +30831,7 @@
           <t>Woodstalker:19</t>
         </is>
       </c>
+      <c r="Z319" t="inlineStr"/>
     </row>
     <row r="320" ht="15" customHeight="1" s="9">
       <c r="A320" s="11" t="n">
@@ -30602,6 +30923,7 @@
           <t>Woodstalker:19</t>
         </is>
       </c>
+      <c r="Z320" t="inlineStr"/>
     </row>
     <row r="321" ht="15" customHeight="1" s="9">
       <c r="A321" s="13" t="n">
@@ -30697,6 +31019,7 @@
           <t>Woodstalker:20</t>
         </is>
       </c>
+      <c r="Z321" t="inlineStr"/>
     </row>
     <row r="322" ht="15" customHeight="1" s="9">
       <c r="A322" s="11" t="n">
@@ -30792,6 +31115,7 @@
           <t>Woodstalker:20</t>
         </is>
       </c>
+      <c r="Z322" t="inlineStr"/>
     </row>
     <row r="323" ht="15" customHeight="1" s="9">
       <c r="A323" s="13" t="n">
@@ -30883,6 +31207,7 @@
           <t>Woodstalker:20</t>
         </is>
       </c>
+      <c r="Z323" t="inlineStr"/>
     </row>
     <row r="324" ht="15" customHeight="1" s="9">
       <c r="A324" s="11" t="n">
@@ -30974,6 +31299,7 @@
           <t>Shadowblade:1</t>
         </is>
       </c>
+      <c r="Z324" t="inlineStr"/>
     </row>
     <row r="325" ht="15" customHeight="1" s="9">
       <c r="A325" s="13" t="n">
@@ -31012,13 +31338,13 @@
         <v>0</v>
       </c>
       <c r="J325" s="13" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K325" s="13" t="n">
         <v>10</v>
       </c>
       <c r="L325" s="13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M325" s="13" t="n">
         <v>5</v>
@@ -31065,6 +31391,7 @@
           <t>Shadowblade:1</t>
         </is>
       </c>
+      <c r="Z325" t="inlineStr"/>
     </row>
     <row r="326" ht="15" customHeight="1" s="9">
       <c r="A326" s="11" t="n">
@@ -31107,13 +31434,13 @@
         <v>6</v>
       </c>
       <c r="J326" s="11" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K326" s="11" t="n">
         <v>10</v>
       </c>
       <c r="L326" s="11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M326" s="11" t="n">
         <v>5</v>
@@ -31160,6 +31487,7 @@
           <t>Shadowblade:2</t>
         </is>
       </c>
+      <c r="Z326" t="inlineStr"/>
     </row>
     <row r="327" ht="15" customHeight="1" s="9">
       <c r="A327" s="13" t="n">
@@ -31198,13 +31526,13 @@
         <v>5</v>
       </c>
       <c r="J327" s="13" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K327" s="13" t="n">
         <v>10</v>
       </c>
       <c r="L327" s="13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M327" s="13" t="n">
         <v>5</v>
@@ -31251,6 +31579,7 @@
           <t>Shadowblade:2</t>
         </is>
       </c>
+      <c r="Z327" t="inlineStr"/>
     </row>
     <row r="328" ht="15" customHeight="1" s="9">
       <c r="A328" s="11" t="n">
@@ -31293,13 +31622,13 @@
         <v>120</v>
       </c>
       <c r="J328" s="11" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K328" s="11" t="n">
         <v>10</v>
       </c>
       <c r="L328" s="11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M328" s="11" t="n">
         <v>5</v>
@@ -31346,6 +31675,7 @@
           <t>Shadowblade:3</t>
         </is>
       </c>
+      <c r="Z328" t="inlineStr"/>
     </row>
     <row r="329" ht="15" customHeight="1" s="9">
       <c r="A329" s="13" t="n">
@@ -31443,6 +31773,7 @@
           <t>Shadowblade:4</t>
         </is>
       </c>
+      <c r="Z329" t="inlineStr"/>
     </row>
     <row r="330" ht="15" customHeight="1" s="9">
       <c r="A330" s="11" t="n">
@@ -31542,6 +31873,7 @@
           <t>Shadowblade:4</t>
         </is>
       </c>
+      <c r="Z330" t="inlineStr"/>
     </row>
     <row r="331" ht="15" customHeight="1" s="9">
       <c r="A331" s="13" t="n">
@@ -31584,13 +31916,13 @@
         <v>15</v>
       </c>
       <c r="J331" s="13" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K331" s="13" t="n">
         <v>10</v>
       </c>
       <c r="L331" s="13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M331" s="13" t="n">
         <v>5</v>
@@ -31639,6 +31971,7 @@
           <t>Shadowblade:5</t>
         </is>
       </c>
+      <c r="Z331" t="inlineStr"/>
     </row>
     <row r="332" ht="15" customHeight="1" s="9">
       <c r="A332" s="11" t="n">
@@ -31681,13 +32014,13 @@
         <v>2</v>
       </c>
       <c r="J332" s="11" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K332" s="11" t="n">
         <v>10</v>
       </c>
       <c r="L332" s="11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M332" s="11" t="n">
         <v>5</v>
@@ -31734,6 +32067,7 @@
           <t>Shadowblade:6</t>
         </is>
       </c>
+      <c r="Z332" t="inlineStr"/>
     </row>
     <row r="333" ht="15" customHeight="1" s="9">
       <c r="A333" s="13" t="n">
@@ -31776,13 +32110,13 @@
         <v>2</v>
       </c>
       <c r="J333" s="13" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K333" s="13" t="n">
         <v>10</v>
       </c>
       <c r="L333" s="13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M333" s="13" t="n">
         <v>5</v>
@@ -31829,6 +32163,7 @@
           <t>Shadowblade:6</t>
         </is>
       </c>
+      <c r="Z333" t="inlineStr"/>
     </row>
     <row r="334" ht="15" customHeight="1" s="9">
       <c r="A334" s="11" t="n">
@@ -31924,6 +32259,7 @@
           <t>Shadowblade:7</t>
         </is>
       </c>
+      <c r="Z334" t="inlineStr"/>
     </row>
     <row r="335" ht="15" customHeight="1" s="9">
       <c r="A335" s="13" t="n">
@@ -32019,6 +32355,7 @@
           <t>Shadowblade:8</t>
         </is>
       </c>
+      <c r="Z335" t="inlineStr"/>
     </row>
     <row r="336" ht="15" customHeight="1" s="9">
       <c r="A336" s="11" t="n">
@@ -32110,6 +32447,7 @@
           <t>Shadowblade:8</t>
         </is>
       </c>
+      <c r="Z336" t="inlineStr"/>
     </row>
     <row r="337" ht="15" customHeight="1" s="9">
       <c r="A337" s="13" t="n">
@@ -32201,6 +32539,7 @@
           <t>Shadowblade:9</t>
         </is>
       </c>
+      <c r="Z337" t="inlineStr"/>
     </row>
     <row r="338" ht="15" customHeight="1" s="9">
       <c r="A338" s="11" t="n">
@@ -32292,6 +32631,7 @@
           <t>Shadowblade:9</t>
         </is>
       </c>
+      <c r="Z338" t="inlineStr"/>
     </row>
     <row r="339" ht="15" customHeight="1" s="9">
       <c r="A339" s="13" t="n">
@@ -32387,6 +32727,7 @@
           <t>Shadowblade:10</t>
         </is>
       </c>
+      <c r="Z339" t="inlineStr"/>
     </row>
     <row r="340" ht="23.85" customHeight="1" s="9">
       <c r="A340" s="11" t="n">
@@ -32484,6 +32825,7 @@
           <t>Shadowblade:11</t>
         </is>
       </c>
+      <c r="Z340" t="inlineStr"/>
     </row>
     <row r="341" ht="15" customHeight="1" s="9">
       <c r="A341" s="13" t="n">
@@ -32575,6 +32917,7 @@
           <t>Shadowblade:11</t>
         </is>
       </c>
+      <c r="Z341" t="inlineStr"/>
     </row>
     <row r="342" ht="15" customHeight="1" s="9">
       <c r="A342" s="11" t="n">
@@ -32666,6 +33009,7 @@
           <t>Shadowblade:12</t>
         </is>
       </c>
+      <c r="Z342" t="inlineStr"/>
     </row>
     <row r="343" ht="15" customHeight="1" s="9">
       <c r="A343" s="13" t="n">
@@ -32763,6 +33107,7 @@
           <t>Shadowblade:12</t>
         </is>
       </c>
+      <c r="Z343" t="inlineStr"/>
     </row>
     <row r="344" ht="15" customHeight="1" s="9">
       <c r="A344" s="11" t="n">
@@ -32854,6 +33199,7 @@
           <t>Shadowblade:13</t>
         </is>
       </c>
+      <c r="Z344" t="inlineStr"/>
     </row>
     <row r="345" ht="15" customHeight="1" s="9">
       <c r="A345" s="13" t="n">
@@ -32949,6 +33295,7 @@
           <t>Shadowblade:13</t>
         </is>
       </c>
+      <c r="Z345" t="inlineStr"/>
     </row>
     <row r="346" ht="15" customHeight="1" s="9">
       <c r="A346" s="11" t="n">
@@ -33044,6 +33391,7 @@
           <t>Shadowblade:14</t>
         </is>
       </c>
+      <c r="Z346" t="inlineStr"/>
     </row>
     <row r="347" ht="15" customHeight="1" s="9">
       <c r="A347" s="13" t="n">
@@ -33145,6 +33493,7 @@
           <t>Shadowblade:15</t>
         </is>
       </c>
+      <c r="Z347" t="inlineStr"/>
     </row>
     <row r="348" ht="15" customHeight="1" s="9">
       <c r="A348" s="11" t="n">
@@ -33236,6 +33585,7 @@
           <t>Shadowblade:15</t>
         </is>
       </c>
+      <c r="Z348" t="inlineStr"/>
     </row>
     <row r="349" ht="15" customHeight="1" s="9">
       <c r="A349" s="13" t="n">
@@ -33331,6 +33681,7 @@
           <t>Shadowblade:16</t>
         </is>
       </c>
+      <c r="Z349" t="inlineStr"/>
     </row>
     <row r="350" ht="15" customHeight="1" s="9">
       <c r="A350" s="11" t="n">
@@ -33426,6 +33777,7 @@
           <t>Shadowblade:16</t>
         </is>
       </c>
+      <c r="Z350" t="inlineStr"/>
     </row>
     <row r="351" ht="15" customHeight="1" s="9">
       <c r="A351" s="13" t="n">
@@ -33521,6 +33873,7 @@
           <t>Shadowblade:17</t>
         </is>
       </c>
+      <c r="Z351" t="inlineStr"/>
     </row>
     <row r="352" ht="15" customHeight="1" s="9">
       <c r="A352" s="11" t="n">
@@ -33618,6 +33971,7 @@
           <t>Shadowblade:17</t>
         </is>
       </c>
+      <c r="Z352" t="inlineStr"/>
     </row>
     <row r="353" ht="15" customHeight="1" s="9">
       <c r="A353" s="13" t="n">
@@ -33709,6 +34063,7 @@
           <t>Shadowblade:18</t>
         </is>
       </c>
+      <c r="Z353" t="inlineStr"/>
     </row>
     <row r="354" ht="15" customHeight="1" s="9">
       <c r="A354" s="11" t="n">
@@ -33806,6 +34161,7 @@
           <t>Shadowblade:18</t>
         </is>
       </c>
+      <c r="Z354" t="inlineStr"/>
     </row>
     <row r="355" ht="15" customHeight="1" s="9">
       <c r="A355" s="13" t="n">
@@ -33901,6 +34257,7 @@
           <t>Shadowblade:19</t>
         </is>
       </c>
+      <c r="Z355" t="inlineStr"/>
     </row>
     <row r="356" ht="15" customHeight="1" s="9">
       <c r="A356" s="11" t="n">
@@ -33998,6 +34355,7 @@
           <t>Shadowblade:19</t>
         </is>
       </c>
+      <c r="Z356" t="inlineStr"/>
     </row>
     <row r="357" ht="15" customHeight="1" s="9">
       <c r="A357" s="13" t="n">
@@ -34093,6 +34451,7 @@
           <t>Shadowblade:20</t>
         </is>
       </c>
+      <c r="Z357" t="inlineStr"/>
     </row>
     <row r="358" ht="15" customHeight="1" s="9">
       <c r="A358" s="11" t="n">
@@ -34184,6 +34543,7 @@
           <t>Shadowblade:20</t>
         </is>
       </c>
+      <c r="Z358" t="inlineStr"/>
     </row>
     <row r="359" ht="23.85" customHeight="1" s="9">
       <c r="A359" s="13" t="n">
@@ -34281,6 +34641,7 @@
           <t>Shadowblade:20</t>
         </is>
       </c>
+      <c r="Z359" t="inlineStr"/>
     </row>
     <row r="360" ht="23.85" customHeight="1" s="9">
       <c r="A360" s="11" t="n">
@@ -34376,6 +34737,11 @@
           <t>Troubadour:1</t>
         </is>
       </c>
+      <c r="Z360" t="inlineStr">
+        <is>
+          <t>The song makes you feel courageous.</t>
+        </is>
+      </c>
     </row>
     <row r="361" ht="15" customHeight="1" s="9">
       <c r="A361" s="13" t="n">
@@ -34471,6 +34837,11 @@
           <t>Troubadour:1</t>
         </is>
       </c>
+      <c r="Z361" t="inlineStr">
+        <is>
+          <t>The dissonant chord's screech makes the enemy wince in pain.</t>
+        </is>
+      </c>
     </row>
     <row r="362" ht="15" customHeight="1" s="9">
       <c r="A362" s="11" t="n">
@@ -34566,6 +34937,11 @@
           <t>Troubadour:2</t>
         </is>
       </c>
+      <c r="Z362" t="inlineStr">
+        <is>
+          <t>Blades of energy assault the nearby enemies.</t>
+        </is>
+      </c>
     </row>
     <row r="363" ht="15" customHeight="1" s="9">
       <c r="A363" s="13" t="n">
@@ -34661,6 +35037,11 @@
           <t>Troubadour:2</t>
         </is>
       </c>
+      <c r="Z363" t="inlineStr">
+        <is>
+          <t>The melody makes the enemy feel strangely at ease.</t>
+        </is>
+      </c>
     </row>
     <row r="364" ht="15" customHeight="1" s="9">
       <c r="A364" s="11" t="n">
@@ -34758,6 +35139,11 @@
           <t>Troubadour:3</t>
         </is>
       </c>
+      <c r="Z364" t="inlineStr">
+        <is>
+          <t>The ballad makes you feel a bit better.</t>
+        </is>
+      </c>
     </row>
     <row r="365" ht="15" customHeight="1" s="9">
       <c r="A365" s="13" t="n">
@@ -34849,6 +35235,7 @@
           <t>Troubadour:4</t>
         </is>
       </c>
+      <c r="Z365" t="inlineStr"/>
     </row>
     <row r="366" ht="15" customHeight="1" s="9">
       <c r="A366" s="11" t="n">
@@ -34940,6 +35327,7 @@
           <t>Troubadour:4</t>
         </is>
       </c>
+      <c r="Z366" t="inlineStr"/>
     </row>
     <row r="367" ht="15" customHeight="1" s="9">
       <c r="A367" s="13" t="n">
@@ -35035,6 +35423,7 @@
           <t>Troubadour:5</t>
         </is>
       </c>
+      <c r="Z367" t="inlineStr"/>
     </row>
     <row r="368" ht="15" customHeight="1" s="9">
       <c r="A368" s="11" t="n">
@@ -35134,6 +35523,7 @@
           <t>Troubadour:6</t>
         </is>
       </c>
+      <c r="Z368" t="inlineStr"/>
     </row>
     <row r="369" ht="15" customHeight="1" s="9">
       <c r="A369" s="13" t="n">
@@ -35229,6 +35619,7 @@
           <t>Troubadour:6</t>
         </is>
       </c>
+      <c r="Z369" t="inlineStr"/>
     </row>
     <row r="370" ht="15" customHeight="1" s="9">
       <c r="A370" s="11" t="n">
@@ -35324,6 +35715,7 @@
           <t>Troubadour:7</t>
         </is>
       </c>
+      <c r="Z370" t="inlineStr"/>
     </row>
     <row r="371" ht="15" customHeight="1" s="9">
       <c r="A371" s="13" t="n">
@@ -35419,6 +35811,7 @@
           <t>Troubadour:8</t>
         </is>
       </c>
+      <c r="Z371" t="inlineStr"/>
     </row>
     <row r="372" ht="15" customHeight="1" s="9">
       <c r="A372" s="11" t="n">
@@ -35514,6 +35907,7 @@
           <t>Troubadour:8</t>
         </is>
       </c>
+      <c r="Z372" t="inlineStr"/>
     </row>
     <row r="373" ht="15" customHeight="1" s="9">
       <c r="A373" s="13" t="n">
@@ -35609,6 +36003,7 @@
           <t>Troubadour:9</t>
         </is>
       </c>
+      <c r="Z373" t="inlineStr"/>
     </row>
     <row r="374" ht="23.85" customHeight="1" s="9">
       <c r="A374" s="11" t="n">
@@ -35700,6 +36095,11 @@
           <t>Troubadour:9</t>
         </is>
       </c>
+      <c r="Z374" t="inlineStr">
+        <is>
+          <t>The song makes you feel courageous.</t>
+        </is>
+      </c>
     </row>
     <row r="375" ht="15" customHeight="1" s="9">
       <c r="A375" s="13" t="n">
@@ -35791,6 +36191,7 @@
           <t>Troubadour:10</t>
         </is>
       </c>
+      <c r="Z375" t="inlineStr"/>
     </row>
     <row r="376" ht="15" customHeight="1" s="9">
       <c r="A376" s="11" t="n">
@@ -35886,6 +36287,7 @@
           <t>Troubadour:11</t>
         </is>
       </c>
+      <c r="Z376" t="inlineStr"/>
     </row>
     <row r="377" ht="15" customHeight="1" s="9">
       <c r="A377" s="13" t="n">
@@ -35981,6 +36383,7 @@
           <t>Troubadour:11</t>
         </is>
       </c>
+      <c r="Z377" t="inlineStr"/>
     </row>
     <row r="378" ht="15" customHeight="1" s="9">
       <c r="A378" s="11" t="n">
@@ -36072,6 +36475,7 @@
           <t>Troubadour:12</t>
         </is>
       </c>
+      <c r="Z378" t="inlineStr"/>
     </row>
     <row r="379" ht="15" customHeight="1" s="9">
       <c r="A379" s="13" t="n">
@@ -36169,6 +36573,7 @@
           <t>Troubadour:12</t>
         </is>
       </c>
+      <c r="Z379" t="inlineStr"/>
     </row>
     <row r="380" ht="15" customHeight="1" s="9">
       <c r="A380" s="11" t="n">
@@ -36351,6 +36756,7 @@
           <t>Troubadour:13</t>
         </is>
       </c>
+      <c r="Z381" t="inlineStr"/>
     </row>
     <row r="382" ht="15" customHeight="1" s="9">
       <c r="A382" s="11" t="n">
@@ -36446,6 +36852,7 @@
           <t>Troubadour:14</t>
         </is>
       </c>
+      <c r="Z382" t="inlineStr"/>
     </row>
     <row r="383" ht="15" customHeight="1" s="9">
       <c r="A383" s="13" t="n">
@@ -36541,6 +36948,7 @@
           <t>Troubadour:15</t>
         </is>
       </c>
+      <c r="Z383" t="inlineStr"/>
     </row>
     <row r="384" ht="15" customHeight="1" s="9">
       <c r="A384" s="11" t="n">
@@ -36636,6 +37044,7 @@
           <t>Troubadour:15</t>
         </is>
       </c>
+      <c r="Z384" t="inlineStr"/>
     </row>
     <row r="385" ht="15" customHeight="1" s="9">
       <c r="A385" s="13" t="n">
@@ -36731,6 +37140,7 @@
           <t>Troubadour:16</t>
         </is>
       </c>
+      <c r="Z385" t="inlineStr"/>
     </row>
     <row r="386" ht="15" customHeight="1" s="9">
       <c r="A386" s="11" t="n">
@@ -36917,6 +37327,7 @@
           <t>Troubadour:17</t>
         </is>
       </c>
+      <c r="Z387" t="inlineStr"/>
     </row>
     <row r="388" ht="15" customHeight="1" s="9">
       <c r="A388" s="11" t="n">
@@ -37012,6 +37423,7 @@
           <t>Troubadour:17</t>
         </is>
       </c>
+      <c r="Z388" t="inlineStr"/>
     </row>
     <row r="389" ht="15" customHeight="1" s="9">
       <c r="A389" s="13" t="n">
@@ -37103,6 +37515,7 @@
           <t>Troubadour:18</t>
         </is>
       </c>
+      <c r="Z389" t="inlineStr"/>
     </row>
     <row r="390" ht="15" customHeight="1" s="9">
       <c r="A390" s="11" t="n">
@@ -37194,6 +37607,7 @@
           <t>Troubadour:18</t>
         </is>
       </c>
+      <c r="Z390" t="inlineStr"/>
     </row>
     <row r="391" ht="15" customHeight="1" s="9">
       <c r="A391" s="13" t="n">
@@ -37289,6 +37703,7 @@
           <t>Troubadour:19</t>
         </is>
       </c>
+      <c r="Z391" t="inlineStr"/>
     </row>
     <row r="392" ht="15" customHeight="1" s="9">
       <c r="A392" s="11" t="n">
@@ -37388,6 +37803,7 @@
           <t>Troubadour:19</t>
         </is>
       </c>
+      <c r="Z392" t="inlineStr"/>
     </row>
     <row r="393" ht="15" customHeight="1" s="9">
       <c r="A393" s="13" t="n">
@@ -37479,6 +37895,7 @@
           <t>Troubadour:20</t>
         </is>
       </c>
+      <c r="Z393" t="inlineStr"/>
     </row>
     <row r="394" ht="15" customHeight="1" s="9">
       <c r="A394" s="11" t="n">
@@ -37574,6 +37991,7 @@
           <t>Troubadour:20</t>
         </is>
       </c>
+      <c r="Z394" t="inlineStr"/>
     </row>
     <row r="395" ht="15" customHeight="1" s="9">
       <c r="A395" s="13" t="n">
@@ -37669,6 +38087,7 @@
           <t>Troubadour:20</t>
         </is>
       </c>
+      <c r="Z395" t="inlineStr"/>
     </row>
     <row r="396" ht="15" customHeight="1" s="9">
       <c r="A396" s="11" t="n">
@@ -37760,6 +38179,7 @@
           <t>Gravecaller:1</t>
         </is>
       </c>
+      <c r="Z396" t="inlineStr"/>
     </row>
     <row r="397" ht="15" customHeight="1" s="9">
       <c r="A397" s="13" t="n">
@@ -37855,6 +38275,11 @@
           <t>Gravecaller:1</t>
         </is>
       </c>
+      <c r="Z397" t="inlineStr">
+        <is>
+          <t>You reanimate a fallen skeleton to serve you.</t>
+        </is>
+      </c>
     </row>
     <row r="398" ht="15" customHeight="1" s="9">
       <c r="A398" s="11" t="n">
@@ -37950,6 +38375,7 @@
           <t>Gravecaller:2</t>
         </is>
       </c>
+      <c r="Z398" t="inlineStr"/>
     </row>
     <row r="399" ht="15" customHeight="1" s="9">
       <c r="A399" s="13" t="n">
@@ -38045,6 +38471,7 @@
           <t>Gravecaller:2</t>
         </is>
       </c>
+      <c r="Z399" t="inlineStr"/>
     </row>
     <row r="400" ht="15" customHeight="1" s="9">
       <c r="A400" s="11" t="n">
@@ -38136,6 +38563,7 @@
           <t>Gravecaller:3</t>
         </is>
       </c>
+      <c r="Z400" t="inlineStr"/>
     </row>
     <row r="401" ht="15" customHeight="1" s="9">
       <c r="A401" s="13" t="n">
@@ -38235,6 +38663,7 @@
           <t>Gravecaller:3</t>
         </is>
       </c>
+      <c r="Z401" t="inlineStr"/>
     </row>
     <row r="402" ht="15" customHeight="1" s="9">
       <c r="A402" s="11" t="n">
@@ -38326,6 +38755,7 @@
           <t>Gravecaller:4</t>
         </is>
       </c>
+      <c r="Z402" t="inlineStr"/>
     </row>
     <row r="403" ht="15" customHeight="1" s="9">
       <c r="A403" s="13" t="n">
@@ -38417,6 +38847,7 @@
           <t>Gravecaller:4</t>
         </is>
       </c>
+      <c r="Z403" t="inlineStr"/>
     </row>
     <row r="404" ht="15" customHeight="1" s="9">
       <c r="A404" s="11" t="n">
@@ -38512,6 +38943,7 @@
           <t>Gravecaller:5</t>
         </is>
       </c>
+      <c r="Z404" t="inlineStr"/>
     </row>
     <row r="405" ht="15" customHeight="1" s="9">
       <c r="A405" s="13" t="n">
@@ -38607,6 +39039,7 @@
           <t>Gravecaller:5</t>
         </is>
       </c>
+      <c r="Z405" t="inlineStr"/>
     </row>
     <row r="406" ht="15" customHeight="1" s="9">
       <c r="A406" s="11" t="n">
@@ -38704,6 +39137,7 @@
           <t>Gravecaller:6</t>
         </is>
       </c>
+      <c r="Z406" t="inlineStr"/>
     </row>
     <row r="407" ht="15" customHeight="1" s="9">
       <c r="A407" s="13" t="n">
@@ -38801,6 +39235,7 @@
           <t>Gravecaller:6</t>
         </is>
       </c>
+      <c r="Z407" t="inlineStr"/>
     </row>
     <row r="408" ht="15" customHeight="1" s="9">
       <c r="A408" s="11" t="n">
@@ -38892,6 +39327,7 @@
           <t>Gravecaller:7</t>
         </is>
       </c>
+      <c r="Z408" t="inlineStr"/>
     </row>
     <row r="409" ht="23.85" customHeight="1" s="9">
       <c r="A409" s="13" t="n">
@@ -38989,6 +39425,7 @@
           <t>Gravecaller:7</t>
         </is>
       </c>
+      <c r="Z409" t="inlineStr"/>
     </row>
     <row r="410" ht="15" customHeight="1" s="9">
       <c r="A410" s="11" t="n">
@@ -39084,6 +39521,7 @@
           <t>Gravecaller:8</t>
         </is>
       </c>
+      <c r="Z410" t="inlineStr"/>
     </row>
     <row r="411" ht="23.85" customHeight="1" s="9">
       <c r="A411" s="13" t="n">
@@ -39179,6 +39617,7 @@
           <t>Gravecaller:8</t>
         </is>
       </c>
+      <c r="Z411" t="inlineStr"/>
     </row>
     <row r="412" ht="15" customHeight="1" s="9">
       <c r="A412" s="11" t="n">
@@ -39270,6 +39709,7 @@
           <t>Gravecaller:9</t>
         </is>
       </c>
+      <c r="Z412" t="inlineStr"/>
     </row>
     <row r="413" ht="15" customHeight="1" s="9">
       <c r="A413" s="13" t="n">
@@ -39361,6 +39801,7 @@
           <t>Gravecaller:9</t>
         </is>
       </c>
+      <c r="Z413" t="inlineStr"/>
     </row>
     <row r="414" ht="15" customHeight="1" s="9">
       <c r="A414" s="11" t="n">
@@ -39456,6 +39897,7 @@
           <t>Gravecaller:10</t>
         </is>
       </c>
+      <c r="Z414" t="inlineStr"/>
     </row>
     <row r="415" ht="23.85" customHeight="1" s="9">
       <c r="A415" s="13" t="n">
@@ -39553,6 +39995,7 @@
           <t>Gravecaller:10</t>
         </is>
       </c>
+      <c r="Z415" t="inlineStr"/>
     </row>
     <row r="416" ht="15" customHeight="1" s="9">
       <c r="A416" s="11" t="n">
@@ -39648,6 +40091,7 @@
           <t>Gravecaller:11</t>
         </is>
       </c>
+      <c r="Z416" t="inlineStr"/>
     </row>
     <row r="417" ht="15" customHeight="1" s="9">
       <c r="A417" s="13" t="n">
@@ -39747,6 +40191,7 @@
           <t>Gravecaller:11</t>
         </is>
       </c>
+      <c r="Z417" t="inlineStr"/>
     </row>
     <row r="418" ht="15" customHeight="1" s="9">
       <c r="A418" s="11" t="n">
@@ -39844,6 +40289,7 @@
           <t>Gravecaller:12</t>
         </is>
       </c>
+      <c r="Z418" t="inlineStr"/>
     </row>
     <row r="419" ht="15" customHeight="1" s="9">
       <c r="A419" s="13" t="n">
@@ -39939,6 +40385,7 @@
           <t>Gravecaller:12</t>
         </is>
       </c>
+      <c r="Z419" t="inlineStr"/>
     </row>
     <row r="420" ht="15" customHeight="1" s="9">
       <c r="A420" s="11" t="n">
@@ -40030,6 +40477,7 @@
           <t>Gravecaller:13</t>
         </is>
       </c>
+      <c r="Z420" t="inlineStr"/>
     </row>
     <row r="421" ht="15" customHeight="1" s="9">
       <c r="A421" s="13" t="n">
@@ -40127,6 +40575,7 @@
           <t>Gravecaller:13</t>
         </is>
       </c>
+      <c r="Z421" t="inlineStr"/>
     </row>
     <row r="422" ht="15" customHeight="1" s="9">
       <c r="A422" s="11" t="n">
@@ -40222,6 +40671,7 @@
           <t>Gravecaller:14</t>
         </is>
       </c>
+      <c r="Z422" t="inlineStr"/>
     </row>
     <row r="423" ht="15" customHeight="1" s="9">
       <c r="A423" s="13" t="n">
@@ -40317,6 +40767,7 @@
           <t>Gravecaller:14</t>
         </is>
       </c>
+      <c r="Z423" t="inlineStr"/>
     </row>
     <row r="424" ht="15" customHeight="1" s="9">
       <c r="A424" s="11" t="n">
@@ -40408,6 +40859,7 @@
           <t>Gravecaller:15</t>
         </is>
       </c>
+      <c r="Z424" t="inlineStr"/>
     </row>
     <row r="425" ht="23.85" customHeight="1" s="9">
       <c r="A425" s="13" t="n">
@@ -40505,6 +40957,7 @@
           <t>Gravecaller:15</t>
         </is>
       </c>
+      <c r="Z425" t="inlineStr"/>
     </row>
     <row r="426" ht="23.85" customHeight="1" s="9">
       <c r="A426" s="11" t="n">
@@ -40602,6 +41055,7 @@
           <t>Gravecaller:16</t>
         </is>
       </c>
+      <c r="Z426" t="inlineStr"/>
     </row>
     <row r="427" ht="23.85" customHeight="1" s="9">
       <c r="A427" s="13" t="n">
@@ -40697,6 +41151,7 @@
           <t>Gravecaller:16</t>
         </is>
       </c>
+      <c r="Z427" t="inlineStr"/>
     </row>
     <row r="428" ht="15" customHeight="1" s="9">
       <c r="A428" s="11" t="n">
@@ -40792,6 +41247,7 @@
           <t>Gravecaller:17</t>
         </is>
       </c>
+      <c r="Z428" t="inlineStr"/>
     </row>
     <row r="429" ht="15" customHeight="1" s="9">
       <c r="A429" s="13" t="n">
@@ -40887,6 +41343,7 @@
           <t>Gravecaller:17</t>
         </is>
       </c>
+      <c r="Z429" t="inlineStr"/>
     </row>
     <row r="430" ht="15" customHeight="1" s="9">
       <c r="A430" s="11" t="n">
@@ -40982,6 +41439,7 @@
           <t>Gravecaller:18</t>
         </is>
       </c>
+      <c r="Z430" t="inlineStr"/>
     </row>
     <row r="431" ht="15" customHeight="1" s="9">
       <c r="A431" s="13" t="n">
@@ -41079,6 +41537,7 @@
           <t>Gravecaller:18</t>
         </is>
       </c>
+      <c r="Z431" t="inlineStr"/>
     </row>
     <row r="432" ht="15" customHeight="1" s="9">
       <c r="A432" s="11" t="n">
@@ -41174,6 +41633,7 @@
           <t>Gravecaller:19</t>
         </is>
       </c>
+      <c r="Z432" t="inlineStr"/>
     </row>
     <row r="433" ht="15" customHeight="1" s="9">
       <c r="A433" s="13" t="n">
@@ -41269,6 +41729,7 @@
           <t>Gravecaller:19</t>
         </is>
       </c>
+      <c r="Z433" t="inlineStr"/>
     </row>
     <row r="434" ht="23.85" customHeight="1" s="9">
       <c r="A434" s="11" t="n">
@@ -41364,6 +41825,7 @@
           <t>Gravecaller:20</t>
         </is>
       </c>
+      <c r="Z434" t="inlineStr"/>
     </row>
     <row r="435" ht="15" customHeight="1" s="9">
       <c r="A435" s="13" t="n">
@@ -41459,6 +41921,7 @@
           <t>Gravecaller:20</t>
         </is>
       </c>
+      <c r="Z435" t="inlineStr"/>
     </row>
     <row r="436" ht="23.85" customHeight="1" s="9">
       <c r="A436" s="11" t="n">
@@ -41554,6 +42017,7 @@
           <t>Gravecaller:20</t>
         </is>
       </c>
+      <c r="Z436" t="inlineStr"/>
     </row>
     <row r="437" ht="15" customHeight="1" s="9">
       <c r="A437" s="13" t="n">
@@ -41649,6 +42113,7 @@
           <t>Runecaster:1</t>
         </is>
       </c>
+      <c r="Z437" t="inlineStr"/>
     </row>
     <row r="438" ht="15" customHeight="1" s="9">
       <c r="A438" s="11" t="n">
@@ -41744,6 +42209,7 @@
           <t>Runecaster:1</t>
         </is>
       </c>
+      <c r="Z438" t="inlineStr"/>
     </row>
     <row r="439" ht="15" customHeight="1" s="9">
       <c r="A439" s="13" t="n">
@@ -41839,6 +42305,7 @@
           <t>Runecaster:2</t>
         </is>
       </c>
+      <c r="Z439" t="inlineStr"/>
     </row>
     <row r="440" ht="15" customHeight="1" s="9">
       <c r="A440" s="11" t="n">
@@ -41930,6 +42397,7 @@
           <t>Arcanist:12, Runecaster:2</t>
         </is>
       </c>
+      <c r="Z440" t="inlineStr"/>
     </row>
     <row r="441" ht="15" customHeight="1" s="9">
       <c r="A441" s="13" t="n">
@@ -42025,6 +42493,7 @@
           <t>Runecaster:3</t>
         </is>
       </c>
+      <c r="Z441" t="inlineStr"/>
     </row>
     <row r="442" ht="15" customHeight="1" s="9">
       <c r="A442" s="11" t="n">
@@ -42116,6 +42585,7 @@
           <t>Runecaster:3</t>
         </is>
       </c>
+      <c r="Z442" t="inlineStr"/>
     </row>
     <row r="443" ht="15" customHeight="1" s="9">
       <c r="A443" s="13" t="n">
@@ -42211,6 +42681,7 @@
           <t>Runecaster:4</t>
         </is>
       </c>
+      <c r="Z443" t="inlineStr"/>
     </row>
     <row r="444" ht="15" customHeight="1" s="9">
       <c r="A444" s="11" t="n">
@@ -42302,6 +42773,7 @@
           <t>Runecaster:4</t>
         </is>
       </c>
+      <c r="Z444" t="inlineStr"/>
     </row>
     <row r="445" ht="15" customHeight="1" s="9">
       <c r="A445" s="13" t="n">
@@ -42397,6 +42869,7 @@
           <t>Runecaster:5</t>
         </is>
       </c>
+      <c r="Z445" t="inlineStr"/>
     </row>
     <row r="446" ht="15" customHeight="1" s="9">
       <c r="A446" s="11" t="n">
@@ -42496,6 +42969,7 @@
           <t>Runecaster:5</t>
         </is>
       </c>
+      <c r="Z446" t="inlineStr"/>
     </row>
     <row r="447" ht="15" customHeight="1" s="9">
       <c r="A447" s="13" t="n">
@@ -42591,6 +43065,7 @@
           <t>Runecaster:6</t>
         </is>
       </c>
+      <c r="Z447" t="inlineStr"/>
     </row>
     <row r="448" ht="15" customHeight="1" s="9">
       <c r="A448" s="11" t="n">
@@ -42686,6 +43161,7 @@
           <t>Runecaster:6</t>
         </is>
       </c>
+      <c r="Z448" t="inlineStr"/>
     </row>
     <row r="449" ht="15" customHeight="1" s="9">
       <c r="A449" s="13" t="n">
@@ -42785,6 +43261,7 @@
           <t>Runecaster:7</t>
         </is>
       </c>
+      <c r="Z449" t="inlineStr"/>
     </row>
     <row r="450" ht="15" customHeight="1" s="9">
       <c r="A450" s="11" t="n">
@@ -42882,6 +43359,7 @@
           <t>Runecaster:7</t>
         </is>
       </c>
+      <c r="Z450" t="inlineStr"/>
     </row>
     <row r="451" ht="15" customHeight="1" s="9">
       <c r="A451" s="13" t="n">
@@ -42973,6 +43451,7 @@
           <t>Runecaster:8</t>
         </is>
       </c>
+      <c r="Z451" t="inlineStr"/>
     </row>
     <row r="452" ht="15" customHeight="1" s="9">
       <c r="A452" s="11" t="n">
@@ -43064,6 +43543,7 @@
           <t>Runecaster:8</t>
         </is>
       </c>
+      <c r="Z452" t="inlineStr"/>
     </row>
     <row r="453" ht="15" customHeight="1" s="9">
       <c r="A453" s="13" t="n">
@@ -43159,6 +43639,7 @@
           <t>Runecaster:9</t>
         </is>
       </c>
+      <c r="Z453" t="inlineStr"/>
     </row>
     <row r="454" ht="15" customHeight="1" s="9">
       <c r="A454" s="11" t="n">
@@ -43254,6 +43735,7 @@
           <t>Runecaster:9</t>
         </is>
       </c>
+      <c r="Z454" t="inlineStr"/>
     </row>
     <row r="455" ht="15" customHeight="1" s="9">
       <c r="A455" s="13" t="n">
@@ -43345,6 +43827,7 @@
           <t>Runecaster:10</t>
         </is>
       </c>
+      <c r="Z455" t="inlineStr"/>
     </row>
     <row r="456" ht="15" customHeight="1" s="9">
       <c r="A456" s="11" t="n">
@@ -43444,6 +43927,7 @@
           <t>Runecaster:10</t>
         </is>
       </c>
+      <c r="Z456" t="inlineStr"/>
     </row>
     <row r="457" ht="15" customHeight="1" s="9">
       <c r="A457" s="13" t="n">
@@ -43535,6 +44019,7 @@
           <t>Runecaster:11</t>
         </is>
       </c>
+      <c r="Z457" t="inlineStr"/>
     </row>
     <row r="458" ht="15" customHeight="1" s="9">
       <c r="A458" s="11" t="n">
@@ -43630,6 +44115,7 @@
           <t>Runecaster:11</t>
         </is>
       </c>
+      <c r="Z458" t="inlineStr"/>
     </row>
     <row r="459" ht="15" customHeight="1" s="9">
       <c r="A459" s="13" t="n">
@@ -43725,6 +44211,7 @@
           <t>Runecaster:12</t>
         </is>
       </c>
+      <c r="Z459" t="inlineStr"/>
     </row>
     <row r="460" ht="15" customHeight="1" s="9">
       <c r="A460" s="11" t="n">
@@ -43820,6 +44307,7 @@
           <t>Runecaster:12</t>
         </is>
       </c>
+      <c r="Z460" t="inlineStr"/>
     </row>
     <row r="461" ht="15" customHeight="1" s="9">
       <c r="A461" s="13" t="n">
@@ -43915,6 +44403,7 @@
           <t>Runecaster:13</t>
         </is>
       </c>
+      <c r="Z461" t="inlineStr"/>
     </row>
     <row r="462" ht="15" customHeight="1" s="9">
       <c r="A462" s="11" t="n">
@@ -44006,6 +44495,7 @@
           <t>Runecaster:13</t>
         </is>
       </c>
+      <c r="Z462" t="inlineStr"/>
     </row>
     <row r="463" ht="15" customHeight="1" s="9">
       <c r="A463" s="13" t="n">
@@ -44101,6 +44591,7 @@
           <t>Runecaster:14</t>
         </is>
       </c>
+      <c r="Z463" t="inlineStr"/>
     </row>
     <row r="464" ht="15" customHeight="1" s="9">
       <c r="A464" s="11" t="n">
@@ -44192,6 +44683,7 @@
           <t>Runecaster:14</t>
         </is>
       </c>
+      <c r="Z464" t="inlineStr"/>
     </row>
     <row r="465" ht="15" customHeight="1" s="9">
       <c r="A465" s="13" t="n">
@@ -44287,6 +44779,7 @@
           <t>Runecaster:15</t>
         </is>
       </c>
+      <c r="Z465" t="inlineStr"/>
     </row>
     <row r="466" ht="15" customHeight="1" s="9">
       <c r="A466" s="11" t="n">
@@ -44378,6 +44871,7 @@
           <t>Runecaster:15</t>
         </is>
       </c>
+      <c r="Z466" t="inlineStr"/>
     </row>
     <row r="467" ht="15" customHeight="1" s="9">
       <c r="A467" s="13" t="n">
@@ -44475,6 +44969,7 @@
           <t>Runecaster:16</t>
         </is>
       </c>
+      <c r="Z467" t="inlineStr"/>
     </row>
     <row r="468" ht="15" customHeight="1" s="9">
       <c r="A468" s="11" t="n">
@@ -44566,6 +45061,7 @@
           <t>Runecaster:16</t>
         </is>
       </c>
+      <c r="Z468" t="inlineStr"/>
     </row>
     <row r="469" ht="15" customHeight="1" s="9">
       <c r="A469" s="13" t="n">
@@ -44657,6 +45153,7 @@
           <t>Runecaster:17</t>
         </is>
       </c>
+      <c r="Z469" t="inlineStr"/>
     </row>
     <row r="470" ht="15" customHeight="1" s="9">
       <c r="A470" s="11" t="n">
@@ -44752,6 +45249,7 @@
           <t>Runecaster:17</t>
         </is>
       </c>
+      <c r="Z470" t="inlineStr"/>
     </row>
     <row r="471" ht="23.85" customHeight="1" s="9">
       <c r="A471" s="13" t="n">
@@ -44843,6 +45341,7 @@
           <t>Runecaster:18</t>
         </is>
       </c>
+      <c r="Z471" t="inlineStr"/>
     </row>
     <row r="472" ht="15" customHeight="1" s="9">
       <c r="A472" s="11" t="n">
@@ -44934,6 +45433,7 @@
           <t>Runecaster:18</t>
         </is>
       </c>
+      <c r="Z472" t="inlineStr"/>
     </row>
     <row r="473" ht="15" customHeight="1" s="9">
       <c r="A473" s="13" t="n">
@@ -45029,6 +45529,7 @@
           <t>Runecaster:19</t>
         </is>
       </c>
+      <c r="Z473" t="inlineStr"/>
     </row>
     <row r="474" ht="15" customHeight="1" s="9">
       <c r="A474" s="11" t="n">
@@ -45128,6 +45629,7 @@
           <t>Runecaster:19</t>
         </is>
       </c>
+      <c r="Z474" t="inlineStr"/>
     </row>
     <row r="475" ht="15" customHeight="1" s="9">
       <c r="A475" s="13" t="n">
@@ -45223,6 +45725,7 @@
           <t>Runecaster:20</t>
         </is>
       </c>
+      <c r="Z475" t="inlineStr"/>
     </row>
     <row r="476" ht="23.85" customHeight="1" s="9">
       <c r="A476" s="11" t="n">
@@ -45318,6 +45821,7 @@
           <t>Runecaster:20</t>
         </is>
       </c>
+      <c r="Z476" t="inlineStr"/>
     </row>
     <row r="477" ht="15" customHeight="1" s="9">
       <c r="A477" s="13" t="n">
@@ -45413,6 +45917,7 @@
           <t>Runecaster:20</t>
         </is>
       </c>
+      <c r="Z477" t="inlineStr"/>
     </row>
     <row r="478" ht="15" customHeight="1" s="9">
       <c r="A478" s="11" t="n">
@@ -45504,6 +46009,7 @@
           <t>Arcanist:1</t>
         </is>
       </c>
+      <c r="Z478" t="inlineStr"/>
     </row>
     <row r="479" ht="15" customHeight="1" s="9">
       <c r="A479" s="13" t="n">
@@ -45595,6 +46101,7 @@
           <t>Arcanist:1</t>
         </is>
       </c>
+      <c r="Z479" t="inlineStr"/>
     </row>
     <row r="480" ht="15" customHeight="1" s="9">
       <c r="A480" s="11" t="n">
@@ -45690,6 +46197,7 @@
           <t>Arcanist:2</t>
         </is>
       </c>
+      <c r="Z480" t="inlineStr"/>
     </row>
     <row r="481" ht="15" customHeight="1" s="9">
       <c r="A481" s="13" t="n">
@@ -45781,6 +46289,7 @@
           <t>Arcanist:2</t>
         </is>
       </c>
+      <c r="Z481" t="inlineStr"/>
     </row>
     <row r="482" ht="15" customHeight="1" s="9">
       <c r="A482" s="11" t="n">
@@ -45872,6 +46381,7 @@
           <t>Arcanist:3</t>
         </is>
       </c>
+      <c r="Z482" t="inlineStr"/>
     </row>
     <row r="483" ht="15" customHeight="1" s="9">
       <c r="A483" s="13" t="n">
@@ -45963,6 +46473,7 @@
           <t>Arcanist:3</t>
         </is>
       </c>
+      <c r="Z483" t="inlineStr"/>
     </row>
     <row r="484" ht="15" customHeight="1" s="9">
       <c r="A484" s="11" t="n">
@@ -46058,6 +46569,7 @@
           <t>Arcanist:4</t>
         </is>
       </c>
+      <c r="Z484" t="inlineStr"/>
     </row>
     <row r="485" ht="15" customHeight="1" s="9">
       <c r="A485" s="13" t="n">
@@ -46153,6 +46665,7 @@
           <t>Arcanist:4</t>
         </is>
       </c>
+      <c r="Z485" t="inlineStr"/>
     </row>
     <row r="486" ht="15" customHeight="1" s="9">
       <c r="A486" s="11" t="n">
@@ -46248,6 +46761,7 @@
           <t>Arcanist:5</t>
         </is>
       </c>
+      <c r="Z486" t="inlineStr"/>
     </row>
     <row r="487" ht="15" customHeight="1" s="9">
       <c r="A487" s="13" t="n">
@@ -46339,6 +46853,7 @@
           <t>Arcanist:5</t>
         </is>
       </c>
+      <c r="Z487" t="inlineStr"/>
     </row>
     <row r="488" ht="15" customHeight="1" s="9">
       <c r="A488" s="11" t="n">
@@ -46434,6 +46949,7 @@
           <t>Arcanist:6</t>
         </is>
       </c>
+      <c r="Z488" t="inlineStr"/>
     </row>
     <row r="489" ht="15" customHeight="1" s="9">
       <c r="A489" s="13" t="n">
@@ -46525,6 +47041,7 @@
           <t>Arcanist:6</t>
         </is>
       </c>
+      <c r="Z489" t="inlineStr"/>
     </row>
     <row r="490" ht="15" customHeight="1" s="9">
       <c r="A490" s="11" t="n">
@@ -46618,6 +47135,7 @@
           <t>Arcanist:7</t>
         </is>
       </c>
+      <c r="Z490" t="inlineStr"/>
     </row>
     <row r="491" ht="15" customHeight="1" s="9">
       <c r="A491" s="13" t="n">
@@ -46709,6 +47227,7 @@
           <t>Arcanist:7</t>
         </is>
       </c>
+      <c r="Z491" t="inlineStr"/>
     </row>
     <row r="492" ht="15" customHeight="1" s="9">
       <c r="A492" s="11" t="n">
@@ -46804,6 +47323,7 @@
           <t>Arcanist:8</t>
         </is>
       </c>
+      <c r="Z492" t="inlineStr"/>
     </row>
     <row r="493" ht="15" customHeight="1" s="9">
       <c r="A493" s="13" t="n">
@@ -46899,6 +47419,7 @@
           <t>Arcanist:8</t>
         </is>
       </c>
+      <c r="Z493" t="inlineStr"/>
     </row>
     <row r="494" ht="15" customHeight="1" s="9">
       <c r="A494" s="11" t="n">
@@ -47081,6 +47602,7 @@
           <t>Arcanist:9</t>
         </is>
       </c>
+      <c r="Z495" t="inlineStr"/>
     </row>
     <row r="496" ht="15" customHeight="1" s="9">
       <c r="A496" s="11" t="n">
@@ -47178,6 +47700,7 @@
           <t>Arcanist:10</t>
         </is>
       </c>
+      <c r="Z496" t="inlineStr"/>
     </row>
     <row r="497" ht="15" customHeight="1" s="9">
       <c r="A497" s="13" t="n">
@@ -47273,6 +47796,7 @@
           <t>Arcanist:10</t>
         </is>
       </c>
+      <c r="Z497" t="inlineStr"/>
     </row>
     <row r="498" ht="15" customHeight="1" s="9">
       <c r="A498" s="11" t="n">
@@ -47372,6 +47896,7 @@
           <t>Arcanist:11</t>
         </is>
       </c>
+      <c r="Z498" t="inlineStr"/>
     </row>
     <row r="499" ht="15" customHeight="1" s="9">
       <c r="A499" s="13" t="n">
@@ -47463,6 +47988,7 @@
           <t>Arcanist:11</t>
         </is>
       </c>
+      <c r="Z499" t="inlineStr"/>
     </row>
     <row r="500" ht="15" customHeight="1" s="9">
       <c r="A500" s="11" t="n">
@@ -47554,6 +48080,7 @@
           <t>Arcanist:12</t>
         </is>
       </c>
+      <c r="Z500" t="inlineStr"/>
     </row>
     <row r="501" ht="15" customHeight="1" s="9">
       <c r="A501" s="13" t="n">
@@ -47649,6 +48176,7 @@
           <t>Arcanist:13</t>
         </is>
       </c>
+      <c r="Z501" t="inlineStr"/>
     </row>
     <row r="502" ht="15" customHeight="1" s="9">
       <c r="A502" s="11" t="n">
@@ -47744,6 +48272,7 @@
           <t>Arcanist:13</t>
         </is>
       </c>
+      <c r="Z502" t="inlineStr"/>
     </row>
     <row r="503" ht="15" customHeight="1" s="9">
       <c r="A503" s="13" t="n">
@@ -47835,6 +48364,7 @@
           <t>Arcanist:14</t>
         </is>
       </c>
+      <c r="Z503" t="inlineStr"/>
     </row>
     <row r="504" ht="15" customHeight="1" s="9">
       <c r="A504" s="11" t="n">
@@ -47930,6 +48460,7 @@
           <t>Arcanist:14</t>
         </is>
       </c>
+      <c r="Z504" t="inlineStr"/>
     </row>
     <row r="505" ht="15" customHeight="1" s="9">
       <c r="A505" s="13" t="n">
@@ -48025,6 +48556,7 @@
           <t>Arcanist:15</t>
         </is>
       </c>
+      <c r="Z505" t="inlineStr"/>
     </row>
     <row r="506" ht="15" customHeight="1" s="9">
       <c r="A506" s="11" t="n">
@@ -48118,6 +48650,7 @@
           <t>Arcanist:15</t>
         </is>
       </c>
+      <c r="Z506" t="inlineStr"/>
     </row>
     <row r="507" ht="23.85" customHeight="1" s="9">
       <c r="A507" s="13" t="n">
@@ -48219,6 +48752,7 @@
           <t>Arcanist:16</t>
         </is>
       </c>
+      <c r="Z507" t="inlineStr"/>
     </row>
     <row r="508" ht="15" customHeight="1" s="9">
       <c r="A508" s="11" t="n">
@@ -48314,6 +48848,7 @@
           <t>Arcanist:16</t>
         </is>
       </c>
+      <c r="Z508" t="inlineStr"/>
     </row>
     <row r="509" ht="15" customHeight="1" s="9">
       <c r="A509" s="13" t="n">
@@ -48409,6 +48944,7 @@
           <t>Arcanist:17</t>
         </is>
       </c>
+      <c r="Z509" t="inlineStr"/>
     </row>
     <row r="510" ht="15" customHeight="1" s="9">
       <c r="A510" s="11" t="n">
@@ -48504,6 +49040,7 @@
           <t>Arcanist:17</t>
         </is>
       </c>
+      <c r="Z510" t="inlineStr"/>
     </row>
     <row r="511" ht="15" customHeight="1" s="9">
       <c r="A511" s="13" t="n">
@@ -48599,6 +49136,7 @@
           <t>Arcanist:18</t>
         </is>
       </c>
+      <c r="Z511" t="inlineStr"/>
     </row>
     <row r="512" ht="15" customHeight="1" s="9">
       <c r="A512" s="11" t="n">
@@ -48690,6 +49228,7 @@
           <t>Arcanist:18</t>
         </is>
       </c>
+      <c r="Z512" t="inlineStr"/>
     </row>
     <row r="513" ht="15" customHeight="1" s="9">
       <c r="A513" s="13" t="n">
@@ -48785,6 +49324,7 @@
           <t>Arcanist:19</t>
         </is>
       </c>
+      <c r="Z513" t="inlineStr"/>
     </row>
     <row r="514" ht="15" customHeight="1" s="9">
       <c r="A514" s="11" t="n">
@@ -48882,6 +49422,7 @@
           <t>Arcanist:19</t>
         </is>
       </c>
+      <c r="Z514" t="inlineStr"/>
     </row>
     <row r="515" ht="15" customHeight="1" s="9">
       <c r="A515" s="13" t="n">
@@ -48981,6 +49522,7 @@
           <t>Arcanist:20</t>
         </is>
       </c>
+      <c r="Z515" t="inlineStr"/>
     </row>
     <row r="516" ht="15" customHeight="1" s="9">
       <c r="A516" s="11" t="n">
@@ -49072,6 +49614,7 @@
           <t>Arcanist:20</t>
         </is>
       </c>
+      <c r="Z516" t="inlineStr"/>
     </row>
     <row r="517" ht="23.85" customHeight="1" s="9">
       <c r="A517" s="13" t="n">
@@ -49163,6 +49706,7 @@
           <t>Wildmage:1</t>
         </is>
       </c>
+      <c r="Z517" t="inlineStr"/>
     </row>
     <row r="518" ht="23.85" customHeight="1" s="9">
       <c r="A518" s="11" t="n">
@@ -49254,6 +49798,7 @@
           <t>Wildmage:1</t>
         </is>
       </c>
+      <c r="Z518" t="inlineStr"/>
     </row>
     <row r="519" ht="23.85" customHeight="1" s="9">
       <c r="A519" s="13" t="n">
@@ -49345,6 +49890,7 @@
           <t>Wildmage:2</t>
         </is>
       </c>
+      <c r="Z519" t="inlineStr"/>
     </row>
     <row r="520" ht="23.85" customHeight="1" s="9">
       <c r="A520" s="11" t="n">
@@ -49440,6 +49986,7 @@
           <t>Wildmage:2</t>
         </is>
       </c>
+      <c r="Z520" t="inlineStr"/>
     </row>
     <row r="521" ht="23.85" customHeight="1" s="9">
       <c r="A521" s="13" t="n">
@@ -49535,6 +50082,7 @@
           <t>Wildmage:3</t>
         </is>
       </c>
+      <c r="Z521" t="inlineStr"/>
     </row>
     <row r="522" ht="23.85" customHeight="1" s="9">
       <c r="A522" s="11" t="n">
@@ -49632,6 +50180,7 @@
           <t>Wildmage:3</t>
         </is>
       </c>
+      <c r="Z522" t="inlineStr"/>
     </row>
     <row r="523" ht="23.85" customHeight="1" s="9">
       <c r="A523" s="13" t="n">
@@ -49723,6 +50272,7 @@
           <t>Wildmage:4</t>
         </is>
       </c>
+      <c r="Z523" t="inlineStr"/>
     </row>
     <row r="524" ht="23.85" customHeight="1" s="9">
       <c r="A524" s="11" t="n">
@@ -49814,6 +50364,7 @@
           <t>Wildmage:4</t>
         </is>
       </c>
+      <c r="Z524" t="inlineStr"/>
     </row>
     <row r="525" ht="23.85" customHeight="1" s="9">
       <c r="A525" s="13" t="n">
@@ -49905,6 +50456,7 @@
           <t>Wildmage:5</t>
         </is>
       </c>
+      <c r="Z525" t="inlineStr"/>
     </row>
     <row r="526" ht="23.85" customHeight="1" s="9">
       <c r="A526" s="11" t="n">
@@ -49996,6 +50548,7 @@
           <t>Wildmage:5</t>
         </is>
       </c>
+      <c r="Z526" t="inlineStr"/>
     </row>
     <row r="527" ht="23.85" customHeight="1" s="9">
       <c r="A527" s="13" t="n">
@@ -50091,6 +50644,7 @@
           <t>Wildmage:6</t>
         </is>
       </c>
+      <c r="Z527" t="inlineStr"/>
     </row>
     <row r="528" ht="23.85" customHeight="1" s="9">
       <c r="A528" s="11" t="n">
@@ -50182,6 +50736,7 @@
           <t>Wildmage:6</t>
         </is>
       </c>
+      <c r="Z528" t="inlineStr"/>
     </row>
     <row r="529" ht="23.85" customHeight="1" s="9">
       <c r="A529" s="13" t="n">
@@ -50273,6 +50828,7 @@
           <t>Wildmage:7</t>
         </is>
       </c>
+      <c r="Z529" t="inlineStr"/>
     </row>
     <row r="530" ht="23.85" customHeight="1" s="9">
       <c r="A530" s="11" t="n">
@@ -50370,6 +50926,7 @@
           <t>Wildmage:7</t>
         </is>
       </c>
+      <c r="Z530" t="inlineStr"/>
     </row>
     <row r="531" ht="23.85" customHeight="1" s="9">
       <c r="A531" s="13" t="n">
@@ -50465,6 +51022,7 @@
           <t>Wildmage:8</t>
         </is>
       </c>
+      <c r="Z531" t="inlineStr"/>
     </row>
     <row r="532" ht="23.85" customHeight="1" s="9">
       <c r="A532" s="11" t="n">
@@ -50560,6 +51118,7 @@
           <t>Wildmage:8</t>
         </is>
       </c>
+      <c r="Z532" t="inlineStr"/>
     </row>
     <row r="533" ht="15" customHeight="1" s="9">
       <c r="A533" s="13" t="n">
@@ -50651,6 +51210,7 @@
           <t>Wildmage:9</t>
         </is>
       </c>
+      <c r="Z533" t="inlineStr"/>
     </row>
     <row r="534" ht="23.85" customHeight="1" s="9">
       <c r="A534" s="11" t="n">
@@ -50742,6 +51302,7 @@
           <t>Wildmage:9</t>
         </is>
       </c>
+      <c r="Z534" t="inlineStr"/>
     </row>
     <row r="535" ht="23.85" customHeight="1" s="9">
       <c r="A535" s="13" t="n">
@@ -50839,6 +51400,7 @@
           <t>Wildmage:10</t>
         </is>
       </c>
+      <c r="Z535" t="inlineStr"/>
     </row>
     <row r="536" ht="23.85" customHeight="1" s="9">
       <c r="A536" s="11" t="n">
@@ -50930,6 +51492,7 @@
           <t>Wildmage:10</t>
         </is>
       </c>
+      <c r="Z536" t="inlineStr"/>
     </row>
     <row r="537" ht="23.85" customHeight="1" s="9">
       <c r="A537" s="13" t="n">
@@ -51025,6 +51588,7 @@
           <t>Wildmage:11</t>
         </is>
       </c>
+      <c r="Z537" t="inlineStr"/>
     </row>
     <row r="538" ht="23.85" customHeight="1" s="9">
       <c r="A538" s="11" t="n">
@@ -51215,6 +51779,7 @@
           <t>Wildmage:12</t>
         </is>
       </c>
+      <c r="Z539" t="inlineStr"/>
     </row>
     <row r="540" ht="23.85" customHeight="1" s="9">
       <c r="A540" s="11" t="n">
@@ -51306,6 +51871,7 @@
           <t>Wildmage:12</t>
         </is>
       </c>
+      <c r="Z540" t="inlineStr"/>
     </row>
     <row r="541" ht="23.85" customHeight="1" s="9">
       <c r="A541" s="13" t="n">
@@ -51397,6 +51963,7 @@
           <t>Wildmage:13</t>
         </is>
       </c>
+      <c r="Z541" t="inlineStr"/>
     </row>
     <row r="542" ht="23.85" customHeight="1" s="9">
       <c r="A542" s="11" t="n">
@@ -51498,6 +52065,7 @@
           <t>Wildmage:13</t>
         </is>
       </c>
+      <c r="Z542" t="inlineStr"/>
     </row>
     <row r="543" ht="23.85" customHeight="1" s="9">
       <c r="A543" s="13" t="n">
@@ -51589,6 +52157,7 @@
           <t>Wildmage:14</t>
         </is>
       </c>
+      <c r="Z543" t="inlineStr"/>
     </row>
     <row r="544" ht="23.85" customHeight="1" s="9">
       <c r="A544" s="11" t="n">
@@ -51686,6 +52255,7 @@
           <t>Wildmage:14</t>
         </is>
       </c>
+      <c r="Z544" t="inlineStr"/>
     </row>
     <row r="545" ht="23.85" customHeight="1" s="9">
       <c r="A545" s="13" t="n">
@@ -51781,6 +52351,7 @@
           <t>Wildmage:15</t>
         </is>
       </c>
+      <c r="Z545" t="inlineStr"/>
     </row>
     <row r="546" ht="23.85" customHeight="1" s="9">
       <c r="A546" s="11" t="n">
@@ -51874,6 +52445,7 @@
           <t>Wildmage:15</t>
         </is>
       </c>
+      <c r="Z546" t="inlineStr"/>
     </row>
     <row r="547" ht="23.85" customHeight="1" s="9">
       <c r="A547" s="13" t="n">
@@ -51971,6 +52543,7 @@
           <t>Wildmage:16</t>
         </is>
       </c>
+      <c r="Z547" t="inlineStr"/>
     </row>
     <row r="548" ht="23.85" customHeight="1" s="9">
       <c r="A548" s="11" t="n">
@@ -52066,6 +52639,7 @@
           <t>Wildmage:16</t>
         </is>
       </c>
+      <c r="Z548" t="inlineStr"/>
     </row>
     <row r="549" ht="23.85" customHeight="1" s="9">
       <c r="A549" s="13" t="n">
@@ -52157,6 +52731,7 @@
           <t>Wildmage:17</t>
         </is>
       </c>
+      <c r="Z549" t="inlineStr"/>
     </row>
     <row r="550" ht="23.85" customHeight="1" s="9">
       <c r="A550" s="11" t="n">
@@ -52248,6 +52823,7 @@
           <t>Wildmage:17</t>
         </is>
       </c>
+      <c r="Z550" t="inlineStr"/>
     </row>
     <row r="551" ht="23.85" customHeight="1" s="9">
       <c r="A551" s="13" t="n">
@@ -52339,6 +52915,7 @@
           <t>Wildmage:18</t>
         </is>
       </c>
+      <c r="Z551" t="inlineStr"/>
     </row>
     <row r="552" ht="23.85" customHeight="1" s="9">
       <c r="A552" s="11" t="n">
@@ -52430,6 +53007,7 @@
           <t>Wildmage:18</t>
         </is>
       </c>
+      <c r="Z552" t="inlineStr"/>
     </row>
     <row r="553" ht="23.85" customHeight="1" s="9">
       <c r="A553" s="13" t="n">
@@ -52525,6 +53103,7 @@
           <t>Wildmage:19</t>
         </is>
       </c>
+      <c r="Z553" t="inlineStr"/>
     </row>
     <row r="554" ht="23.85" customHeight="1" s="9">
       <c r="A554" s="11" t="n">
@@ -52616,6 +53195,7 @@
           <t>Wildmage:19</t>
         </is>
       </c>
+      <c r="Z554" t="inlineStr"/>
     </row>
     <row r="555" ht="23.85" customHeight="1" s="9">
       <c r="A555" s="13" t="n">
@@ -52711,6 +53291,7 @@
           <t>Wildmage:20</t>
         </is>
       </c>
+      <c r="Z555" t="inlineStr"/>
     </row>
     <row r="556" ht="23.85" customHeight="1" s="9">
       <c r="A556" s="11" t="n">
@@ -52806,6 +53387,7 @@
           <t>Wildmage:20</t>
         </is>
       </c>
+      <c r="Z556" t="inlineStr"/>
     </row>
     <row r="557" ht="23.85" customHeight="1" s="9">
       <c r="A557" s="13" t="n">
@@ -52903,6 +53485,7 @@
           <t>Wildmage:20</t>
         </is>
       </c>
+      <c r="Z557" t="inlineStr"/>
     </row>
     <row r="558" ht="15" customHeight="1" s="9">
       <c r="A558" s="11" t="n">
@@ -52998,6 +53581,7 @@
           <t>Voidknight:2</t>
         </is>
       </c>
+      <c r="Z558" t="inlineStr"/>
     </row>
     <row r="559" ht="23.85" customHeight="1" s="9">
       <c r="A559" s="13" t="n">
@@ -53093,6 +53677,7 @@
           <t>Voidknight:8</t>
         </is>
       </c>
+      <c r="Z559" t="inlineStr"/>
     </row>
     <row r="560" ht="23.85" customHeight="1" s="9">
       <c r="A560" s="11" t="n">
@@ -53188,6 +53773,7 @@
           <t>Blademaster:1, Lightsworn:1, Voidknight:1</t>
         </is>
       </c>
+      <c r="Z560" t="inlineStr"/>
     </row>
     <row r="561" ht="35.05" customHeight="1" s="9">
       <c r="A561" s="13" t="n">
@@ -53283,6 +53869,100 @@
       <c r="Y561" s="14" t="inlineStr">
         <is>
           <t>Spiritcaller:1</t>
+        </is>
+      </c>
+      <c r="Z561" t="inlineStr"/>
+    </row>
+    <row r="562">
+      <c r="A562" t="n">
+        <v>585</v>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>blindside</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>A quick blow to the head that stuns the target for 3 seconds: long enough to slip behind it for a Backstab.</t>
+        </is>
+      </c>
+      <c r="D562" t="n">
+        <v>1</v>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>physical</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>detrimental</t>
+        </is>
+      </c>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>stun</t>
+        </is>
+      </c>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="I562" t="n">
+        <v>10</v>
+      </c>
+      <c r="J562" t="n">
+        <v>0</v>
+      </c>
+      <c r="K562" t="n">
+        <v>20</v>
+      </c>
+      <c r="L562" t="n">
+        <v>0</v>
+      </c>
+      <c r="M562" t="n">
+        <v>3</v>
+      </c>
+      <c r="N562" t="inlineStr">
+        <is>
+          <t>3m</t>
+        </is>
+      </c>
+      <c r="P562" t="b">
+        <v>0</v>
+      </c>
+      <c r="S562" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="T562" t="n">
+        <v>0</v>
+      </c>
+      <c r="U562" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="V562" t="b">
+        <v>1</v>
+      </c>
+      <c r="W562" t="b">
+        <v>1</v>
+      </c>
+      <c r="X562" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y562" t="inlineStr">
+        <is>
+          <t>Shadowblade:1</t>
+        </is>
+      </c>
+      <c r="Z562" t="inlineStr">
+        <is>
+          <t>You crack $targetname across the head. $Targetname reels, stunned!</t>
         </is>
       </c>
     </row>

</xml_diff>